<commit_message>
guitar tom anderson 追加
</commit_message>
<xml_diff>
--- a/_docs/設計メモ.xlsx
+++ b/_docs/設計メモ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repository\portfolio\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2734A29-1FA6-49B3-B24B-0E50C3599CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAC2DD5E-CF3F-4F65-8E31-9A773FE55C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" tabRatio="778" firstSheet="2" activeTab="3" xr2:uid="{23010AEC-8D3D-48D3-938D-B3932852B25B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="778" firstSheet="2" activeTab="3" xr2:uid="{23010AEC-8D3D-48D3-938D-B3932852B25B}"/>
   </bookViews>
   <sheets>
     <sheet name="architecture" sheetId="12" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4852" uniqueCount="2453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4856" uniqueCount="2454">
   <si>
     <t>状態異常</t>
     <rPh sb="0" eb="2">
@@ -10222,6 +10222,10 @@
   </si>
   <si>
     <t>https://killer.jp/index.html</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>TOM ANDERSON</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -15274,8 +15278,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7911971" y="1528349"/>
-          <a:ext cx="1800328" cy="1214718"/>
+          <a:off x="7985930" y="1467837"/>
+          <a:ext cx="1820498" cy="1167653"/>
           <a:chOff x="8992083" y="208776"/>
           <a:chExt cx="1814762" cy="1244600"/>
         </a:xfrm>
@@ -15584,8 +15588,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="11175520" y="3059605"/>
-          <a:ext cx="1822530" cy="1963728"/>
+          <a:off x="11283097" y="2938582"/>
+          <a:ext cx="1842700" cy="1889768"/>
           <a:chOff x="8549484" y="3956874"/>
           <a:chExt cx="1810288" cy="1437363"/>
         </a:xfrm>
@@ -16136,8 +16140,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4681098" y="1657961"/>
-          <a:ext cx="1869953" cy="3342717"/>
+          <a:off x="4721439" y="1597449"/>
+          <a:ext cx="1890124" cy="3208246"/>
           <a:chOff x="5970441" y="628674"/>
           <a:chExt cx="1893913" cy="3428095"/>
         </a:xfrm>
@@ -16605,8 +16609,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="10840271" y="7258650"/>
-          <a:ext cx="2193307" cy="2523422"/>
+          <a:off x="10941124" y="6969538"/>
+          <a:ext cx="2220201" cy="2422569"/>
           <a:chOff x="12007370" y="5957071"/>
           <a:chExt cx="2223130" cy="2581251"/>
         </a:xfrm>
@@ -16812,8 +16816,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="14334233" y="4816236"/>
-          <a:ext cx="2220036" cy="1720343"/>
+          <a:off x="14468704" y="4627977"/>
+          <a:ext cx="2246929" cy="1653108"/>
           <a:chOff x="15050343" y="4729843"/>
           <a:chExt cx="2243515" cy="1763032"/>
         </a:xfrm>
@@ -17242,8 +17246,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="6846794" y="5210735"/>
-          <a:ext cx="1781735" cy="1311089"/>
+          <a:off x="6914030" y="5002306"/>
+          <a:ext cx="1795181" cy="1264024"/>
           <a:chOff x="6846794" y="5210735"/>
           <a:chExt cx="2341399" cy="1311089"/>
         </a:xfrm>
@@ -17619,8 +17623,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="3726679" y="7642890"/>
-          <a:ext cx="2335072" cy="1882107"/>
+          <a:off x="3760297" y="7340331"/>
+          <a:ext cx="2355242" cy="1808149"/>
           <a:chOff x="3726679" y="7642891"/>
           <a:chExt cx="2335072" cy="1468663"/>
         </a:xfrm>
@@ -18543,15 +18547,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6672014-33B5-48C4-9202-55E4E667EEEF}">
   <dimension ref="A1:W32"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="3.75" customWidth="1"/>
-    <col min="2" max="3" width="8.75" customWidth="1"/>
-    <col min="20" max="21" width="2.75" customWidth="1"/>
-    <col min="22" max="23" width="4.125" customWidth="1"/>
-    <col min="24" max="24" width="4.75" customWidth="1"/>
-    <col min="25" max="25" width="8.75" customWidth="1"/>
-    <col min="27" max="27" width="4.375" customWidth="1"/>
+    <col min="1" max="1" width="3.69921875" customWidth="1"/>
+    <col min="2" max="3" width="8.69921875" customWidth="1"/>
+    <col min="20" max="21" width="2.69921875" customWidth="1"/>
+    <col min="22" max="23" width="4.09765625" customWidth="1"/>
+    <col min="24" max="24" width="4.69921875" customWidth="1"/>
+    <col min="25" max="25" width="8.69921875" customWidth="1"/>
+    <col min="27" max="27" width="4.3984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -18559,25 +18563,25 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="20.25">
+    <row r="2" spans="1:23" ht="19.2">
       <c r="A2" s="108"/>
       <c r="B2" s="107" t="s">
         <v>1931</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="20.25">
+    <row r="3" spans="1:23" ht="19.2">
       <c r="A3" s="107"/>
       <c r="B3" s="107" t="s">
         <v>1932</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="20.25">
+    <row r="4" spans="1:23" ht="19.2">
       <c r="A4" s="107"/>
       <c r="B4" s="107" t="s">
         <v>1933</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="19.5" thickBot="1">
+    <row r="5" spans="1:23" ht="18.600000000000001" thickBot="1">
       <c r="V5" s="67"/>
       <c r="W5" s="67"/>
     </row>
@@ -18611,7 +18615,7 @@
       <c r="C8" s="64"/>
       <c r="W8" s="65"/>
     </row>
-    <row r="9" spans="1:23" ht="19.5" thickBot="1">
+    <row r="9" spans="1:23" ht="18.600000000000001" thickBot="1">
       <c r="C9" s="64"/>
       <c r="L9" t="s">
         <v>1706</v>
@@ -18761,7 +18765,7 @@
       <c r="V30" s="65"/>
       <c r="W30" s="65"/>
     </row>
-    <row r="31" spans="3:23" ht="19.5" thickBot="1">
+    <row r="31" spans="3:23" ht="18.600000000000001" thickBot="1">
       <c r="C31" s="64"/>
       <c r="D31" s="66"/>
       <c r="E31" s="67"/>
@@ -18784,7 +18788,7 @@
       <c r="V31" s="68"/>
       <c r="W31" s="65"/>
     </row>
-    <row r="32" spans="3:23" ht="13.15" customHeight="1" thickBot="1">
+    <row r="32" spans="3:23" ht="13.2" customHeight="1" thickBot="1">
       <c r="C32" s="66"/>
       <c r="D32" s="67"/>
       <c r="E32" s="67"/>
@@ -18817,10 +18821,10 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC349EE6-5475-4F9C-BD43-5DC02797CE07}">
   <dimension ref="A2:R415"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="1" width="11" style="98" customWidth="1"/>
-    <col min="2" max="6" width="10.875" style="98" customWidth="1"/>
+    <col min="2" max="6" width="10.8984375" style="98" customWidth="1"/>
     <col min="7" max="16384" width="9" style="98"/>
   </cols>
   <sheetData>
@@ -21282,10 +21286,10 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71F0B575-2DDF-49B9-8DE2-F372EEC2F3B3}">
   <dimension ref="A2:O139"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.6"/>
   <cols>
-    <col min="1" max="1" width="11.875" style="1" customWidth="1"/>
-    <col min="2" max="6" width="10.875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.8984375" style="1" customWidth="1"/>
+    <col min="2" max="6" width="10.8984375" style="1" customWidth="1"/>
     <col min="7" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -21317,7 +21321,7 @@
         <v>1537</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="18.75">
+    <row r="4" spans="1:15" ht="18">
       <c r="A4" s="1" t="s">
         <v>1280</v>
       </c>
@@ -21346,7 +21350,7 @@
         <v>1539</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" ht="13.2">
       <c r="B5" s="58" t="s">
         <v>1175</v>
       </c>
@@ -21363,7 +21367,7 @@
         <v>1292</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" ht="13.2">
       <c r="B6" s="58" t="s">
         <v>1176</v>
       </c>
@@ -21386,7 +21390,7 @@
         <v>1370</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" ht="13.2">
       <c r="B7" s="58" t="s">
         <v>1189</v>
       </c>
@@ -21415,7 +21419,7 @@
         <v>1555</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" ht="13.2">
       <c r="B8" s="58" t="s">
         <v>1177</v>
       </c>
@@ -21444,7 +21448,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" ht="13.2">
       <c r="B9" s="58" t="s">
         <v>1178</v>
       </c>
@@ -21470,7 +21474,7 @@
         <v>1557</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" ht="13.2">
       <c r="B10" s="58" t="s">
         <v>1179</v>
       </c>
@@ -21496,7 +21500,7 @@
         <v>1382</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" ht="13.2">
       <c r="B11" s="58" t="s">
         <v>1180</v>
       </c>
@@ -21522,7 +21526,7 @@
         <v>1383</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" ht="13.2">
       <c r="B12" s="58" t="s">
         <v>1181</v>
       </c>
@@ -21548,7 +21552,7 @@
         <v>1384</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" ht="13.2">
       <c r="B13" s="58" t="s">
         <v>1182</v>
       </c>
@@ -21571,7 +21575,7 @@
         <v>1187</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" ht="13.2">
       <c r="B14" s="58" t="s">
         <v>1183</v>
       </c>
@@ -21594,7 +21598,7 @@
         <v>1385</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" ht="13.2">
       <c r="B15" s="58" t="s">
         <v>1184</v>
       </c>
@@ -21617,7 +21621,7 @@
         <v>1371</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" ht="13.2">
       <c r="B16" s="58" t="s">
         <v>1185</v>
       </c>
@@ -21637,7 +21641,7 @@
         <v>1372</v>
       </c>
     </row>
-    <row r="17" spans="2:10">
+    <row r="17" spans="2:10" ht="13.2">
       <c r="B17" s="58" t="s">
         <v>1186</v>
       </c>
@@ -21657,7 +21661,7 @@
         <v>1207</v>
       </c>
     </row>
-    <row r="18" spans="2:10">
+    <row r="18" spans="2:10" ht="13.2">
       <c r="B18" s="58" t="s">
         <v>1190</v>
       </c>
@@ -21677,7 +21681,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="19" spans="2:10">
+    <row r="19" spans="2:10" ht="13.2">
       <c r="B19" s="58" t="s">
         <v>1187</v>
       </c>
@@ -21697,7 +21701,7 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="20" spans="2:10">
+    <row r="20" spans="2:10" ht="13.2">
       <c r="B20" s="58" t="s">
         <v>1191</v>
       </c>
@@ -22550,7 +22554,7 @@
         <v>2381</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="18.75">
+    <row r="112" spans="1:7" ht="18">
       <c r="A112" s="1" t="s">
         <v>2439</v>
       </c>
@@ -22573,7 +22577,7 @@
         <v>2385</v>
       </c>
     </row>
-    <row r="113" spans="2:7" ht="18.75">
+    <row r="113" spans="2:7" ht="18">
       <c r="B113" s="111" t="s">
         <v>2386</v>
       </c>
@@ -22593,7 +22597,7 @@
         <v>2388</v>
       </c>
     </row>
-    <row r="114" spans="2:7" ht="18.75">
+    <row r="114" spans="2:7" ht="18">
       <c r="B114" s="111" t="s">
         <v>2389</v>
       </c>
@@ -22613,7 +22617,7 @@
         <v>2390</v>
       </c>
     </row>
-    <row r="115" spans="2:7" ht="18.75">
+    <row r="115" spans="2:7" ht="18">
       <c r="B115" s="111" t="s">
         <v>2391</v>
       </c>
@@ -22633,7 +22637,7 @@
         <v>2393</v>
       </c>
     </row>
-    <row r="116" spans="2:7" ht="18.75">
+    <row r="116" spans="2:7" ht="18">
       <c r="B116" s="111" t="s">
         <v>2394</v>
       </c>
@@ -22653,7 +22657,7 @@
         <v>2395</v>
       </c>
     </row>
-    <row r="117" spans="2:7" ht="18.75">
+    <row r="117" spans="2:7" ht="18">
       <c r="B117" s="111" t="s">
         <v>2396</v>
       </c>
@@ -22673,7 +22677,7 @@
         <v>2397</v>
       </c>
     </row>
-    <row r="118" spans="2:7" ht="18.75">
+    <row r="118" spans="2:7" ht="18">
       <c r="B118" s="111" t="s">
         <v>2398</v>
       </c>
@@ -22693,7 +22697,7 @@
         <v>2399</v>
       </c>
     </row>
-    <row r="119" spans="2:7" ht="18.75">
+    <row r="119" spans="2:7" ht="18">
       <c r="B119" s="111" t="s">
         <v>2369</v>
       </c>
@@ -22733,7 +22737,7 @@
         <v>2403</v>
       </c>
     </row>
-    <row r="121" spans="2:7" ht="18.75">
+    <row r="121" spans="2:7" ht="18">
       <c r="B121" s="111" t="s">
         <v>2404</v>
       </c>
@@ -22753,7 +22757,7 @@
         <v>2405</v>
       </c>
     </row>
-    <row r="122" spans="2:7" ht="18.75">
+    <row r="122" spans="2:7" ht="18">
       <c r="B122" s="111" t="s">
         <v>2406</v>
       </c>
@@ -22773,7 +22777,7 @@
         <v>2407</v>
       </c>
     </row>
-    <row r="123" spans="2:7" ht="18.75">
+    <row r="123" spans="2:7" ht="18">
       <c r="B123" s="111" t="s">
         <v>2375</v>
       </c>
@@ -22793,7 +22797,7 @@
         <v>2408</v>
       </c>
     </row>
-    <row r="124" spans="2:7" ht="18.75">
+    <row r="124" spans="2:7" ht="18">
       <c r="B124" s="111" t="s">
         <v>2409</v>
       </c>
@@ -22813,7 +22817,7 @@
         <v>2410</v>
       </c>
     </row>
-    <row r="125" spans="2:7" ht="18.75">
+    <row r="125" spans="2:7" ht="18">
       <c r="B125" s="111" t="s">
         <v>2411</v>
       </c>
@@ -22833,7 +22837,7 @@
         <v>2412</v>
       </c>
     </row>
-    <row r="126" spans="2:7" ht="18.75">
+    <row r="126" spans="2:7" ht="18">
       <c r="B126" s="111" t="s">
         <v>2413</v>
       </c>
@@ -22853,7 +22857,7 @@
         <v>2414</v>
       </c>
     </row>
-    <row r="127" spans="2:7" ht="18.75">
+    <row r="127" spans="2:7" ht="18">
       <c r="B127" s="111" t="s">
         <v>2441</v>
       </c>
@@ -22873,7 +22877,7 @@
         <v>2415</v>
       </c>
     </row>
-    <row r="128" spans="2:7" ht="18.75">
+    <row r="128" spans="2:7" ht="18">
       <c r="B128" s="111" t="s">
         <v>2416</v>
       </c>
@@ -22893,7 +22897,7 @@
         <v>2417</v>
       </c>
     </row>
-    <row r="129" spans="2:7" ht="18.75">
+    <row r="129" spans="2:7" ht="18">
       <c r="B129" s="111" t="s">
         <v>2325</v>
       </c>
@@ -22913,7 +22917,7 @@
         <v>2418</v>
       </c>
     </row>
-    <row r="130" spans="2:7" ht="18.75">
+    <row r="130" spans="2:7" ht="18">
       <c r="B130" s="111" t="s">
         <v>2419</v>
       </c>
@@ -22933,7 +22937,7 @@
         <v>2420</v>
       </c>
     </row>
-    <row r="131" spans="2:7" ht="18.75">
+    <row r="131" spans="2:7" ht="18">
       <c r="B131" s="111" t="s">
         <v>2421</v>
       </c>
@@ -22953,7 +22957,7 @@
         <v>2422</v>
       </c>
     </row>
-    <row r="132" spans="2:7" ht="18.75">
+    <row r="132" spans="2:7" ht="18">
       <c r="B132" s="111" t="s">
         <v>2423</v>
       </c>
@@ -22973,7 +22977,7 @@
         <v>2425</v>
       </c>
     </row>
-    <row r="133" spans="2:7" ht="18.75">
+    <row r="133" spans="2:7" ht="18">
       <c r="B133" s="111" t="s">
         <v>2426</v>
       </c>
@@ -22993,7 +22997,7 @@
         <v>2427</v>
       </c>
     </row>
-    <row r="134" spans="2:7" ht="18.75">
+    <row r="134" spans="2:7" ht="18">
       <c r="B134" s="111" t="s">
         <v>2428</v>
       </c>
@@ -23013,7 +23017,7 @@
         <v>2429</v>
       </c>
     </row>
-    <row r="135" spans="2:7" ht="18.75">
+    <row r="135" spans="2:7" ht="18">
       <c r="B135" s="111" t="s">
         <v>2430</v>
       </c>
@@ -23033,7 +23037,7 @@
         <v>2431</v>
       </c>
     </row>
-    <row r="136" spans="2:7" ht="18.75">
+    <row r="136" spans="2:7" ht="18">
       <c r="B136" s="111" t="s">
         <v>2338</v>
       </c>
@@ -23053,7 +23057,7 @@
         <v>2432</v>
       </c>
     </row>
-    <row r="137" spans="2:7" ht="18.75">
+    <row r="137" spans="2:7" ht="18">
       <c r="B137" s="111" t="s">
         <v>2433</v>
       </c>
@@ -23073,7 +23077,7 @@
         <v>2434</v>
       </c>
     </row>
-    <row r="138" spans="2:7" ht="18.75">
+    <row r="138" spans="2:7" ht="18">
       <c r="B138" s="111" t="s">
         <v>2435</v>
       </c>
@@ -23093,7 +23097,7 @@
         <v>2436</v>
       </c>
     </row>
-    <row r="139" spans="2:7" ht="18.75">
+    <row r="139" spans="2:7" ht="18">
       <c r="B139" s="111" t="s">
         <v>2437</v>
       </c>
@@ -23130,9 +23134,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46FCFD5C-696C-43AD-A2BD-D69C05CB2D44}">
   <dimension ref="B2:P57"/>
-  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="12.6"/>
   <cols>
-    <col min="1" max="16384" width="8.75" style="1"/>
+    <col min="1" max="16384" width="8.69921875" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:16">
@@ -23608,9 +23612,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E898285-845A-4583-B20D-F3A331C07E8E}">
   <dimension ref="B2:R45"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
-    <col min="13" max="13" width="8.625" customWidth="1"/>
+    <col min="13" max="13" width="8.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:18">
@@ -23625,7 +23629,7 @@
       <c r="O2" s="86"/>
       <c r="P2" s="86"/>
     </row>
-    <row r="3" spans="2:18" ht="19.5" thickBot="1">
+    <row r="3" spans="2:18" ht="18.600000000000001" thickBot="1">
       <c r="F3" s="89" t="s">
         <v>1582</v>
       </c>
@@ -23747,7 +23751,7 @@
       <c r="P10" s="65"/>
       <c r="R10" s="84"/>
     </row>
-    <row r="11" spans="2:18" ht="19.5" thickBot="1">
+    <row r="11" spans="2:18" ht="18.600000000000001" thickBot="1">
       <c r="F11" s="91"/>
       <c r="I11" s="75"/>
       <c r="J11" s="66"/>
@@ -23836,7 +23840,7 @@
         <v>1686</v>
       </c>
     </row>
-    <row r="22" spans="4:18" ht="19.5" thickBot="1">
+    <row r="22" spans="4:18" ht="18.600000000000001" thickBot="1">
       <c r="D22" s="80"/>
       <c r="E22" s="81"/>
       <c r="F22" s="81"/>
@@ -23965,7 +23969,7 @@
       </c>
       <c r="N29" s="84"/>
     </row>
-    <row r="30" spans="4:18" ht="19.5" thickBot="1">
+    <row r="30" spans="4:18" ht="18.600000000000001" thickBot="1">
       <c r="D30" s="83"/>
       <c r="E30" s="77"/>
       <c r="F30" s="78"/>
@@ -24201,11 +24205,11 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD79B98E-03E4-44E6-9FBF-39CA1C89C95A}">
   <dimension ref="B3:L149"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
-    <col min="2" max="2" width="8.75" style="73"/>
-    <col min="3" max="3" width="10.625" customWidth="1"/>
-    <col min="6" max="6" width="10.875" customWidth="1"/>
+    <col min="2" max="2" width="8.69921875" style="73"/>
+    <col min="3" max="3" width="10.59765625" customWidth="1"/>
+    <col min="6" max="6" width="10.8984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:10">
@@ -24985,7 +24989,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="16384" width="9" style="5"/>
   </cols>
@@ -24999,7 +25003,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EBD988A-503C-4F44-AC4A-B26683FC9B4C}">
   <dimension ref="B4:O34"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="16384" width="9" style="5"/>
   </cols>
@@ -25149,15 +25153,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B38E66FE-6CF0-4EAE-97A5-1587F7EEF1C8}">
-  <dimension ref="B4:K175"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <dimension ref="B4:K176"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="1" width="9" style="5"/>
-    <col min="2" max="2" width="20.25" style="5" customWidth="1"/>
-    <col min="3" max="3" width="24.125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.19921875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="24.09765625" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17" style="5" customWidth="1"/>
     <col min="5" max="8" width="9" style="5"/>
-    <col min="9" max="9" width="45.625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="45.59765625" style="5" customWidth="1"/>
     <col min="10" max="22" width="9" style="5"/>
     <col min="23" max="23" width="8" style="5" customWidth="1"/>
     <col min="24" max="16384" width="9" style="5"/>
@@ -27762,7 +27766,7 @@
         <v>1551</v>
       </c>
       <c r="K102" s="5" t="str">
-        <f t="shared" ref="K102:K113" si="14">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B102&amp;"'"&amp;","&amp;E102&amp;","&amp;"'"&amp;C102&amp;"'"&amp;","&amp;"'"&amp;D102&amp;"'"&amp;","&amp;"'"&amp;F102&amp;"'"&amp;","&amp;G102&amp;","&amp;H102&amp;","&amp;"'"&amp;I102&amp;"'"&amp;");"</f>
+        <f t="shared" ref="K102:K114" si="14">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B102&amp;"'"&amp;","&amp;E102&amp;","&amp;"'"&amp;C102&amp;"'"&amp;","&amp;"'"&amp;D102&amp;"'"&amp;","&amp;"'"&amp;F102&amp;"'"&amp;","&amp;G102&amp;","&amp;H102&amp;","&amp;"'"&amp;I102&amp;"'"&amp;");"</f>
         <v>INSERT INTO m_code VALUES ('guitar_makers',10,'MusicMan','','',0,0.0,'https://www.music-man.com/instruments/guitars');</v>
       </c>
     </row>
@@ -27814,7 +27818,7 @@
         <v>1553</v>
       </c>
       <c r="K104" s="5" t="str">
-        <f t="shared" ref="K104:K112" si="15">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B104&amp;"'"&amp;","&amp;E104&amp;","&amp;"'"&amp;C104&amp;"'"&amp;","&amp;"'"&amp;D104&amp;"'"&amp;","&amp;"'"&amp;F104&amp;"'"&amp;","&amp;G104&amp;","&amp;H104&amp;","&amp;"'"&amp;I104&amp;"'"&amp;");"</f>
+        <f t="shared" ref="K104:K113" si="15">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B104&amp;"'"&amp;","&amp;E104&amp;","&amp;"'"&amp;C104&amp;"'"&amp;","&amp;"'"&amp;D104&amp;"'"&amp;","&amp;"'"&amp;F104&amp;"'"&amp;","&amp;G104&amp;","&amp;H104&amp;","&amp;"'"&amp;I104&amp;"'"&amp;");"</f>
         <v>INSERT INTO m_code VALUES ('guitar_makers',12,'Momose','','',0,0.0,'https://www.deviser.co.jp/momose');</v>
       </c>
     </row>
@@ -28048,62 +28052,60 @@
         <v>2452</v>
       </c>
       <c r="K113" s="5" t="str">
+        <f t="shared" si="15"/>
+        <v>INSERT INTO m_code VALUES ('guitar_makers',21,'Killer','','',0,0.0,'https://killer.jp/index.html');</v>
+      </c>
+    </row>
+    <row r="114" spans="2:11">
+      <c r="B114" s="8" t="s">
+        <v>1777</v>
+      </c>
+      <c r="C114" s="8" t="s">
+        <v>2453</v>
+      </c>
+      <c r="D114" s="8"/>
+      <c r="E114" s="8">
+        <v>22</v>
+      </c>
+      <c r="F114" s="8"/>
+      <c r="G114" s="9">
+        <v>0</v>
+      </c>
+      <c r="H114" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="I114" s="8" t="s">
+        <v>2452</v>
+      </c>
+      <c r="K114" s="5" t="str">
         <f t="shared" si="14"/>
-        <v>INSERT INTO m_code VALUES ('guitar_makers',21,'Killer','','',0,0.0,'https://killer.jp/index.html');</v>
-      </c>
-    </row>
-    <row r="114" spans="2:11">
-      <c r="B114" s="6" t="s">
+        <v>INSERT INTO m_code VALUES ('guitar_makers',22,'TOM ANDERSON','','',0,0.0,'https://killer.jp/index.html');</v>
+      </c>
+    </row>
+    <row r="115" spans="2:11">
+      <c r="B115" s="6" t="s">
         <v>1542</v>
       </c>
-      <c r="C114" s="6" t="s">
+      <c r="C115" s="6" t="s">
         <v>1388</v>
       </c>
-      <c r="D114" s="6" t="s">
+      <c r="D115" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="E114" s="7" t="s">
+      <c r="E115" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="F114" s="6" t="s">
+      <c r="F115" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="G114" s="6" t="s">
+      <c r="G115" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="H114" s="6" t="s">
+      <c r="H115" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="I114" s="6" t="s">
+      <c r="I115" s="6" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="115" spans="2:11">
-      <c r="B115" s="8" t="s">
-        <v>1778</v>
-      </c>
-      <c r="C115" s="8" t="s">
-        <v>1425</v>
-      </c>
-      <c r="D115" s="8"/>
-      <c r="E115" s="8">
-        <v>1</v>
-      </c>
-      <c r="F115" s="8" t="s">
-        <v>1439</v>
-      </c>
-      <c r="G115" s="9">
-        <v>0</v>
-      </c>
-      <c r="H115" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="I115" s="8" t="s">
-        <v>1463</v>
-      </c>
-      <c r="K115" s="5" t="str">
-        <f t="shared" ref="K115:K150" si="16">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B115&amp;"'"&amp;","&amp;E115&amp;","&amp;"'"&amp;C115&amp;"'"&amp;","&amp;"'"&amp;D115&amp;"'"&amp;","&amp;"'"&amp;F115&amp;"'"&amp;","&amp;G115&amp;","&amp;H115&amp;","&amp;"'"&amp;I115&amp;"'"&amp;");"</f>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',1,'HardMaple','','ハードメイプル',0,0.0,'硬質でタイト、明瞭なアタック。');</v>
       </c>
     </row>
     <row r="116" spans="2:11">
@@ -28111,14 +28113,14 @@
         <v>1778</v>
       </c>
       <c r="C116" s="8" t="s">
-        <v>1426</v>
+        <v>1425</v>
       </c>
       <c r="D116" s="8"/>
       <c r="E116" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F116" s="8" t="s">
-        <v>1440</v>
+        <v>1439</v>
       </c>
       <c r="G116" s="9">
         <v>0</v>
@@ -28127,11 +28129,11 @@
         <v>125</v>
       </c>
       <c r="I116" s="8" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="K116" s="5" t="str">
-        <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',2,'FlameMaple','','フレイムメイプル',0,0.0,'明るく抜けが良く、華やかな倍音。');</v>
+        <f t="shared" ref="K116:K151" si="16">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B116&amp;"'"&amp;","&amp;E116&amp;","&amp;"'"&amp;C116&amp;"'"&amp;","&amp;"'"&amp;D116&amp;"'"&amp;","&amp;"'"&amp;F116&amp;"'"&amp;","&amp;G116&amp;","&amp;H116&amp;","&amp;"'"&amp;I116&amp;"'"&amp;");"</f>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',1,'HardMaple','','ハードメイプル',0,0.0,'硬質でタイト、明瞭なアタック。');</v>
       </c>
     </row>
     <row r="117" spans="2:11">
@@ -28139,14 +28141,14 @@
         <v>1778</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>1427</v>
+        <v>1426</v>
       </c>
       <c r="D117" s="8"/>
       <c r="E117" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F117" s="8" t="s">
-        <v>1441</v>
+        <v>1440</v>
       </c>
       <c r="G117" s="9">
         <v>0</v>
@@ -28155,11 +28157,11 @@
         <v>125</v>
       </c>
       <c r="I117" s="8" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
       <c r="K117" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',3,'QuiltedMaple','','キルテッドメイプル',0,0.0,'立体的で広がりがあり、煌びやかな響き。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',2,'FlameMaple','','フレイムメイプル',0,0.0,'明るく抜けが良く、華やかな倍音。');</v>
       </c>
     </row>
     <row r="118" spans="2:11">
@@ -28167,14 +28169,14 @@
         <v>1778</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>1428</v>
+        <v>1427</v>
       </c>
       <c r="D118" s="8"/>
       <c r="E118" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F118" s="8" t="s">
-        <v>1442</v>
+        <v>1441</v>
       </c>
       <c r="G118" s="9">
         <v>0</v>
@@ -28183,11 +28185,11 @@
         <v>125</v>
       </c>
       <c r="I118" s="8" t="s">
-        <v>1466</v>
+        <v>1465</v>
       </c>
       <c r="K118" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',4,'BirdseyeMaple','','バーズアイメイプル',0,0.0,'粒立ちが良く、明るくシャープ。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',3,'QuiltedMaple','','キルテッドメイプル',0,0.0,'立体的で広がりがあり、煌びやかな響き。');</v>
       </c>
     </row>
     <row r="119" spans="2:11">
@@ -28195,14 +28197,14 @@
         <v>1778</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>1429</v>
+        <v>1428</v>
       </c>
       <c r="D119" s="8"/>
       <c r="E119" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F119" s="8" t="s">
-        <v>1443</v>
+        <v>1442</v>
       </c>
       <c r="G119" s="9">
         <v>0</v>
@@ -28211,11 +28213,11 @@
         <v>125</v>
       </c>
       <c r="I119" s="8" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
       <c r="K119" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',5,'RoastedMaple','','ローステッドメイプル',0,0.0,'引き締まったタイトな音で反応が速い。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',4,'BirdseyeMaple','','バーズアイメイプル',0,0.0,'粒立ちが良く、明るくシャープ。');</v>
       </c>
     </row>
     <row r="120" spans="2:11">
@@ -28223,14 +28225,14 @@
         <v>1778</v>
       </c>
       <c r="C120" s="8" t="s">
-        <v>1389</v>
+        <v>1429</v>
       </c>
       <c r="D120" s="8"/>
       <c r="E120" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F120" s="8" t="s">
-        <v>1438</v>
+        <v>1443</v>
       </c>
       <c r="G120" s="9">
         <v>0</v>
@@ -28239,11 +28241,11 @@
         <v>125</v>
       </c>
       <c r="I120" s="8" t="s">
-        <v>1462</v>
+        <v>1467</v>
       </c>
       <c r="K120" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',6,'Maple','','メイプル',0,0.0,'明るくハリがあり、アタックが強い。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',5,'RoastedMaple','','ローステッドメイプル',0,0.0,'引き締まったタイトな音で反応が速い。');</v>
       </c>
     </row>
     <row r="121" spans="2:11">
@@ -28251,14 +28253,14 @@
         <v>1778</v>
       </c>
       <c r="C121" s="8" t="s">
-        <v>1430</v>
+        <v>1389</v>
       </c>
       <c r="D121" s="8"/>
       <c r="E121" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F121" s="8" t="s">
-        <v>1444</v>
+        <v>1438</v>
       </c>
       <c r="G121" s="9">
         <v>0</v>
@@ -28267,11 +28269,11 @@
         <v>125</v>
       </c>
       <c r="I121" s="8" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
       <c r="K121" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',7,'HonduranMahogany','','ホンジュラスマホガニー',0,0.0,'深みがあり、太くリッチな中低域。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',6,'Maple','','メイプル',0,0.0,'明るくハリがあり、アタックが強い。');</v>
       </c>
     </row>
     <row r="122" spans="2:11">
@@ -28279,14 +28281,14 @@
         <v>1778</v>
       </c>
       <c r="C122" s="8" t="s">
-        <v>1390</v>
+        <v>1430</v>
       </c>
       <c r="D122" s="8"/>
       <c r="E122" s="8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F122" s="8" t="s">
-        <v>1408</v>
+        <v>1444</v>
       </c>
       <c r="G122" s="9">
         <v>0</v>
@@ -28295,11 +28297,11 @@
         <v>125</v>
       </c>
       <c r="I122" s="8" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
       <c r="K122" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',8,'Mahogany','','マホガニー',0,0.0,'中低域が豊かで温かい音。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',7,'HonduranMahogany','','ホンジュラスマホガニー',0,0.0,'深みがあり、太くリッチな中低域。');</v>
       </c>
     </row>
     <row r="123" spans="2:11">
@@ -28307,14 +28309,14 @@
         <v>1778</v>
       </c>
       <c r="C123" s="8" t="s">
-        <v>1431</v>
+        <v>1390</v>
       </c>
       <c r="D123" s="8"/>
       <c r="E123" s="8">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F123" s="8" t="s">
-        <v>1445</v>
+        <v>1408</v>
       </c>
       <c r="G123" s="9">
         <v>0</v>
@@ -28323,11 +28325,11 @@
         <v>125</v>
       </c>
       <c r="I123" s="8" t="s">
-        <v>1470</v>
+        <v>1468</v>
       </c>
       <c r="K123" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',9,'Sapele','','サペリ',0,0.0,'温かく柔らかいトーンでバランスが良い。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',8,'Mahogany','','マホガニー',0,0.0,'中低域が豊かで温かい音。');</v>
       </c>
     </row>
     <row r="124" spans="2:11">
@@ -28335,14 +28337,14 @@
         <v>1778</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>1397</v>
+        <v>1431</v>
       </c>
       <c r="D124" s="8"/>
       <c r="E124" s="8">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F124" s="8" t="s">
-        <v>1446</v>
+        <v>1445</v>
       </c>
       <c r="G124" s="9">
         <v>0</v>
@@ -28351,11 +28353,11 @@
         <v>125</v>
       </c>
       <c r="I124" s="8" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
       <c r="K124" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',10,'Korina','','コリーナ',0,0.0,'中域が豊かで太い音。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',9,'Sapele','','サペリ',0,0.0,'温かく柔らかいトーンでバランスが良い。');</v>
       </c>
     </row>
     <row r="125" spans="2:11">
@@ -28363,14 +28365,14 @@
         <v>1778</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>1432</v>
+        <v>1397</v>
       </c>
       <c r="D125" s="8"/>
       <c r="E125" s="8">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F125" s="8" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
       <c r="G125" s="9">
         <v>0</v>
@@ -28379,11 +28381,11 @@
         <v>125</v>
       </c>
       <c r="I125" s="8" t="s">
-        <v>1472</v>
+        <v>1471</v>
       </c>
       <c r="K125" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',11,'WhiteKorina','','ホワイトコリーナ',0,0.0,'明るく抜けが良く、軽快なレスポンス。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',10,'Korina','','コリーナ',0,0.0,'中域が豊かで太い音。');</v>
       </c>
     </row>
     <row r="126" spans="2:11">
@@ -28391,14 +28393,14 @@
         <v>1778</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>1391</v>
+        <v>1432</v>
       </c>
       <c r="D126" s="8"/>
       <c r="E126" s="8">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F126" s="8" t="s">
-        <v>1409</v>
+        <v>1447</v>
       </c>
       <c r="G126" s="9">
         <v>0</v>
@@ -28407,11 +28409,11 @@
         <v>125</v>
       </c>
       <c r="I126" s="8" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="K126" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',12,'Alder','','アルダー',0,0.0,'バランスが良くクセが少ない。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',11,'WhiteKorina','','ホワイトコリーナ',0,0.0,'明るく抜けが良く、軽快なレスポンス。');</v>
       </c>
     </row>
     <row r="127" spans="2:11">
@@ -28419,14 +28421,14 @@
         <v>1778</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>1392</v>
+        <v>1391</v>
       </c>
       <c r="D127" s="8"/>
       <c r="E127" s="8">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F127" s="8" t="s">
-        <v>1448</v>
+        <v>1409</v>
       </c>
       <c r="G127" s="9">
         <v>0</v>
@@ -28435,11 +28437,11 @@
         <v>125</v>
       </c>
       <c r="I127" s="8" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
       <c r="K127" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',13,'Ash','','アッシュ',0,0.0,'明るく抜ける音でアタックが強い。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',12,'Alder','','アルダー',0,0.0,'バランスが良くクセが少ない。');</v>
       </c>
     </row>
     <row r="128" spans="2:11">
@@ -28447,14 +28449,14 @@
         <v>1778</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>1393</v>
+        <v>1392</v>
       </c>
       <c r="D128" s="8"/>
       <c r="E128" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F128" s="8" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="G128" s="9">
         <v>0</v>
@@ -28463,11 +28465,11 @@
         <v>125</v>
       </c>
       <c r="I128" s="8" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="K128" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',14,'Basswood','','バスウッド',0,0.0,'軽く柔らかく、ウォームで扱いやすい。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',13,'Ash','','アッシュ',0,0.0,'明るく抜ける音でアタックが強い。');</v>
       </c>
     </row>
     <row r="129" spans="2:11">
@@ -28475,14 +28477,14 @@
         <v>1778</v>
       </c>
       <c r="C129" s="8" t="s">
-        <v>1402</v>
+        <v>1393</v>
       </c>
       <c r="D129" s="8"/>
       <c r="E129" s="8">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F129" s="8" t="s">
-        <v>1450</v>
+        <v>1449</v>
       </c>
       <c r="G129" s="9">
         <v>0</v>
@@ -28491,11 +28493,11 @@
         <v>125</v>
       </c>
       <c r="I129" s="8" t="s">
-        <v>1476</v>
+        <v>1475</v>
       </c>
       <c r="K129" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',15,'Poplar','','ポプラ',0,0.0,'軽く素直でクセが少ない。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',14,'Basswood','','バスウッド',0,0.0,'軽く柔らかく、ウォームで扱いやすい。');</v>
       </c>
     </row>
     <row r="130" spans="2:11">
@@ -28503,14 +28505,14 @@
         <v>1778</v>
       </c>
       <c r="C130" s="8" t="s">
-        <v>1398</v>
+        <v>1402</v>
       </c>
       <c r="D130" s="8"/>
       <c r="E130" s="8">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F130" s="8" t="s">
-        <v>1451</v>
+        <v>1450</v>
       </c>
       <c r="G130" s="9">
         <v>0</v>
@@ -28519,11 +28521,11 @@
         <v>125</v>
       </c>
       <c r="I130" s="8" t="s">
-        <v>1477</v>
+        <v>1476</v>
       </c>
       <c r="K130" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',16,'Spruce','','スプルース',0,0.0,'軽く響きが良く、明るいトーン。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',15,'Poplar','','ポプラ',0,0.0,'軽く素直でクセが少ない。');</v>
       </c>
     </row>
     <row r="131" spans="2:11">
@@ -28531,14 +28533,14 @@
         <v>1778</v>
       </c>
       <c r="C131" s="8" t="s">
-        <v>1399</v>
+        <v>1398</v>
       </c>
       <c r="D131" s="8"/>
       <c r="E131" s="8">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F131" s="8" t="s">
-        <v>1452</v>
+        <v>1451</v>
       </c>
       <c r="G131" s="9">
         <v>0</v>
@@ -28547,11 +28549,11 @@
         <v>125</v>
       </c>
       <c r="I131" s="8" t="s">
-        <v>1478</v>
+        <v>1477</v>
       </c>
       <c r="K131" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',17,'Cedar','','シダー',0,0.0,'柔らかく温かい音。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',16,'Spruce','','スプルース',0,0.0,'軽く響きが良く、明るいトーン。');</v>
       </c>
     </row>
     <row r="132" spans="2:11">
@@ -28559,14 +28561,14 @@
         <v>1778</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>1433</v>
+        <v>1399</v>
       </c>
       <c r="D132" s="8"/>
       <c r="E132" s="8">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F132" s="8" t="s">
-        <v>1454</v>
+        <v>1452</v>
       </c>
       <c r="G132" s="9">
         <v>0</v>
@@ -28575,11 +28577,11 @@
         <v>125</v>
       </c>
       <c r="I132" s="8" t="s">
-        <v>1480</v>
+        <v>1478</v>
       </c>
       <c r="K132" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',18,'IndianRosewood','','インディアンローズウッド',0,0.0,'甘く深みがあり、豊かな中低域。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',17,'Cedar','','シダー',0,0.0,'柔らかく温かい音。');</v>
       </c>
     </row>
     <row r="133" spans="2:11">
@@ -28587,14 +28589,14 @@
         <v>1778</v>
       </c>
       <c r="C133" s="8" t="s">
-        <v>1434</v>
+        <v>1433</v>
       </c>
       <c r="D133" s="8"/>
       <c r="E133" s="8">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F133" s="8" t="s">
-        <v>1455</v>
+        <v>1454</v>
       </c>
       <c r="G133" s="9">
         <v>0</v>
@@ -28603,11 +28605,11 @@
         <v>125</v>
       </c>
       <c r="I133" s="8" t="s">
-        <v>1481</v>
+        <v>1480</v>
       </c>
       <c r="K133" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',19,'BrazilianRosewood','','ブラジリアンローズウッド',0,0.0,'濃厚で深いトーン、豊かな倍音。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',18,'IndianRosewood','','インディアンローズウッド',0,0.0,'甘く深みがあり、豊かな中低域。');</v>
       </c>
     </row>
     <row r="134" spans="2:11">
@@ -28615,14 +28617,14 @@
         <v>1778</v>
       </c>
       <c r="C134" s="8" t="s">
-        <v>1394</v>
+        <v>1434</v>
       </c>
       <c r="D134" s="8"/>
       <c r="E134" s="8">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F134" s="8" t="s">
-        <v>1453</v>
+        <v>1455</v>
       </c>
       <c r="G134" s="9">
         <v>0</v>
@@ -28631,11 +28633,11 @@
         <v>125</v>
       </c>
       <c r="I134" s="8" t="s">
-        <v>1479</v>
+        <v>1481</v>
       </c>
       <c r="K134" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',20,'Rosewood','','ローズウッド',0,0.0,'甘く丸い音で中域が豊か。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',19,'BrazilianRosewood','','ブラジリアンローズウッド',0,0.0,'濃厚で深いトーン、豊かな倍音。');</v>
       </c>
     </row>
     <row r="135" spans="2:11">
@@ -28643,14 +28645,14 @@
         <v>1778</v>
       </c>
       <c r="C135" s="8" t="s">
-        <v>1435</v>
+        <v>1394</v>
       </c>
       <c r="D135" s="8"/>
       <c r="E135" s="8">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F135" s="8" t="s">
-        <v>1410</v>
+        <v>1453</v>
       </c>
       <c r="G135" s="9">
         <v>0</v>
@@ -28659,11 +28661,11 @@
         <v>125</v>
       </c>
       <c r="I135" s="8" t="s">
-        <v>1482</v>
+        <v>1479</v>
       </c>
       <c r="K135" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',21,'PauFerro','','パーフェロー',0,0.0,'明るく硬質でタイトな音。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',20,'Rosewood','','ローズウッド',0,0.0,'甘く丸い音で中域が豊か。');</v>
       </c>
     </row>
     <row r="136" spans="2:11">
@@ -28671,14 +28673,14 @@
         <v>1778</v>
       </c>
       <c r="C136" s="8" t="s">
-        <v>1400</v>
+        <v>1435</v>
       </c>
       <c r="D136" s="8"/>
       <c r="E136" s="8">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F136" s="8" t="s">
-        <v>1411</v>
+        <v>1410</v>
       </c>
       <c r="G136" s="9">
         <v>0</v>
@@ -28687,11 +28689,11 @@
         <v>125</v>
       </c>
       <c r="I136" s="8" t="s">
-        <v>1483</v>
+        <v>1482</v>
       </c>
       <c r="K136" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',22,'Ovangkol','','オバンコール',0,0.0,'中域が豊かで温かいトーン。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',21,'PauFerro','','パーフェロー',0,0.0,'明るく硬質でタイトな音。');</v>
       </c>
     </row>
     <row r="137" spans="2:11">
@@ -28699,14 +28701,14 @@
         <v>1778</v>
       </c>
       <c r="C137" s="8" t="s">
-        <v>1395</v>
+        <v>1400</v>
       </c>
       <c r="D137" s="8"/>
       <c r="E137" s="8">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F137" s="8" t="s">
-        <v>1456</v>
+        <v>1411</v>
       </c>
       <c r="G137" s="9">
         <v>0</v>
@@ -28715,11 +28717,11 @@
         <v>125</v>
       </c>
       <c r="I137" s="8" t="s">
-        <v>1484</v>
+        <v>1483</v>
       </c>
       <c r="K137" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',23,'Ebony','','エボニー',0,0.0,'硬くタイトで高域がクリア。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',22,'Ovangkol','','オバンコール',0,0.0,'中域が豊かで温かいトーン。');</v>
       </c>
     </row>
     <row r="138" spans="2:11">
@@ -28727,14 +28729,14 @@
         <v>1778</v>
       </c>
       <c r="C138" s="8" t="s">
-        <v>1396</v>
+        <v>1395</v>
       </c>
       <c r="D138" s="8"/>
       <c r="E138" s="8">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F138" s="8" t="s">
-        <v>1457</v>
+        <v>1456</v>
       </c>
       <c r="G138" s="9">
         <v>0</v>
@@ -28743,11 +28745,11 @@
         <v>125</v>
       </c>
       <c r="I138" s="8" t="s">
-        <v>1416</v>
+        <v>1484</v>
       </c>
       <c r="K138" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',24,'Walnut','','ウォルナット',0,0.0,'中域が豊かで落ち着いたトーン。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',23,'Ebony','','エボニー',0,0.0,'硬くタイトで高域がクリア。');</v>
       </c>
     </row>
     <row r="139" spans="2:11">
@@ -28755,14 +28757,14 @@
         <v>1778</v>
       </c>
       <c r="C139" s="8" t="s">
-        <v>1436</v>
+        <v>1396</v>
       </c>
       <c r="D139" s="8"/>
       <c r="E139" s="8">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F139" s="8" t="s">
-        <v>1458</v>
+        <v>1457</v>
       </c>
       <c r="G139" s="9">
         <v>0</v>
@@ -28771,11 +28773,11 @@
         <v>125</v>
       </c>
       <c r="I139" s="8" t="s">
-        <v>1485</v>
+        <v>1416</v>
       </c>
       <c r="K139" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',25,'Padauk','','パドゥーク',0,0.0,'明るく抜けが良く、個性的な響き。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',24,'Walnut','','ウォルナット',0,0.0,'中域が豊かで落ち着いたトーン。');</v>
       </c>
     </row>
     <row r="140" spans="2:11">
@@ -28783,14 +28785,14 @@
         <v>1778</v>
       </c>
       <c r="C140" s="8" t="s">
-        <v>1401</v>
+        <v>1436</v>
       </c>
       <c r="D140" s="8"/>
       <c r="E140" s="8">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F140" s="8" t="s">
-        <v>1459</v>
+        <v>1458</v>
       </c>
       <c r="G140" s="9">
         <v>0</v>
@@ -28799,11 +28801,11 @@
         <v>125</v>
       </c>
       <c r="I140" s="8" t="s">
-        <v>1486</v>
+        <v>1485</v>
       </c>
       <c r="K140" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',26,'Koa','','コア',0,0.0,'明るく華やかで軽快。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',25,'Padauk','','パドゥーク',0,0.0,'明るく抜けが良く、個性的な響き。');</v>
       </c>
     </row>
     <row r="141" spans="2:11">
@@ -28811,14 +28813,14 @@
         <v>1778</v>
       </c>
       <c r="C141" s="8" t="s">
-        <v>1403</v>
+        <v>1401</v>
       </c>
       <c r="D141" s="8"/>
       <c r="E141" s="8">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F141" s="8" t="s">
-        <v>1460</v>
+        <v>1459</v>
       </c>
       <c r="G141" s="9">
         <v>0</v>
@@ -28827,11 +28829,11 @@
         <v>125</v>
       </c>
       <c r="I141" s="8" t="s">
-        <v>1487</v>
+        <v>1486</v>
       </c>
       <c r="K141" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',27,'Nato','','ナトー',0,0.0,'中低域が豊かで温かい。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',26,'Koa','','コア',0,0.0,'明るく華やかで軽快。');</v>
       </c>
     </row>
     <row r="142" spans="2:11">
@@ -28839,14 +28841,14 @@
         <v>1778</v>
       </c>
       <c r="C142" s="8" t="s">
-        <v>1404</v>
+        <v>1403</v>
       </c>
       <c r="D142" s="8"/>
       <c r="E142" s="8">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F142" s="8" t="s">
-        <v>1412</v>
+        <v>1460</v>
       </c>
       <c r="G142" s="9">
         <v>0</v>
@@ -28855,11 +28857,11 @@
         <v>125</v>
       </c>
       <c r="I142" s="8" t="s">
-        <v>1488</v>
+        <v>1487</v>
       </c>
       <c r="K142" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',28,'Agathis','','アガチス',0,0.0,'柔らかくウォームで素直。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',27,'Nato','','ナトー',0,0.0,'中低域が豊かで温かい。');</v>
       </c>
     </row>
     <row r="143" spans="2:11">
@@ -28867,14 +28869,14 @@
         <v>1778</v>
       </c>
       <c r="C143" s="8" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="D143" s="8"/>
       <c r="E143" s="8">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F143" s="8" t="s">
-        <v>1413</v>
+        <v>1412</v>
       </c>
       <c r="G143" s="9">
         <v>0</v>
@@ -28883,11 +28885,11 @@
         <v>125</v>
       </c>
       <c r="I143" s="8" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
       <c r="K143" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',29,'Bubinga','','ブビンガ',0,0.0,'重く硬質でサスティンが長い。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',28,'Agathis','','アガチス',0,0.0,'柔らかくウォームで素直。');</v>
       </c>
     </row>
     <row r="144" spans="2:11">
@@ -28895,14 +28897,14 @@
         <v>1778</v>
       </c>
       <c r="C144" s="8" t="s">
-        <v>1406</v>
+        <v>1405</v>
       </c>
       <c r="D144" s="8"/>
       <c r="E144" s="8">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F144" s="8" t="s">
-        <v>1414</v>
+        <v>1413</v>
       </c>
       <c r="G144" s="9">
         <v>0</v>
@@ -28911,11 +28913,11 @@
         <v>125</v>
       </c>
       <c r="I144" s="8" t="s">
-        <v>1490</v>
+        <v>1489</v>
       </c>
       <c r="K144" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',30,'Wenge','','ウェンジ',0,0.0,'非常に硬くタイトで個性的。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',29,'Bubinga','','ブビンガ',0,0.0,'重く硬質でサスティンが長い。');</v>
       </c>
     </row>
     <row r="145" spans="2:11">
@@ -28923,14 +28925,14 @@
         <v>1778</v>
       </c>
       <c r="C145" s="8" t="s">
-        <v>1407</v>
+        <v>1406</v>
       </c>
       <c r="D145" s="8"/>
       <c r="E145" s="8">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F145" s="8" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="G145" s="9">
         <v>0</v>
@@ -28939,11 +28941,11 @@
         <v>125</v>
       </c>
       <c r="I145" s="8" t="s">
-        <v>1491</v>
+        <v>1490</v>
       </c>
       <c r="K145" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',31,'Purpleheart','','パープルハート',0,0.0,'硬く鮮やかでアタックが強い。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',30,'Wenge','','ウェンジ',0,0.0,'非常に硬くタイトで個性的。');</v>
       </c>
     </row>
     <row r="146" spans="2:11">
@@ -28951,14 +28953,14 @@
         <v>1778</v>
       </c>
       <c r="C146" s="8" t="s">
-        <v>1437</v>
+        <v>1407</v>
       </c>
       <c r="D146" s="8"/>
       <c r="E146" s="8">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F146" s="8" t="s">
-        <v>1461</v>
+        <v>1415</v>
       </c>
       <c r="G146" s="9">
         <v>0</v>
@@ -28967,11 +28969,11 @@
         <v>125</v>
       </c>
       <c r="I146" s="8" t="s">
-        <v>1492</v>
+        <v>1491</v>
       </c>
       <c r="K146" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',32,'Zebrawood','','ゼブラウッド',0,0.0,'明るく硬質でクセのあるトーン。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',31,'Purpleheart','','パープルハート',0,0.0,'硬く鮮やかでアタックが強い。');</v>
       </c>
     </row>
     <row r="147" spans="2:11">
@@ -28979,14 +28981,14 @@
         <v>1778</v>
       </c>
       <c r="C147" s="8" t="s">
-        <v>1558</v>
+        <v>1437</v>
       </c>
       <c r="D147" s="8"/>
       <c r="E147" s="8">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F147" s="8" t="s">
-        <v>1559</v>
+        <v>1461</v>
       </c>
       <c r="G147" s="9">
         <v>0</v>
@@ -28995,11 +28997,11 @@
         <v>125</v>
       </c>
       <c r="I147" s="8" t="s">
-        <v>1560</v>
+        <v>1492</v>
       </c>
       <c r="K147" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',33,'Okoume','','オクメ',0,0.0,'マホガニーに近く、中低域が豊かで軽量。');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',32,'Zebrawood','','ゼブラウッド',0,0.0,'明るく硬質でクセのあるトーン。');</v>
       </c>
     </row>
     <row r="148" spans="2:11">
@@ -29007,14 +29009,14 @@
         <v>1778</v>
       </c>
       <c r="C148" s="8" t="s">
-        <v>1562</v>
+        <v>1558</v>
       </c>
       <c r="D148" s="8"/>
       <c r="E148" s="8">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F148" s="8" t="s">
-        <v>1561</v>
+        <v>1559</v>
       </c>
       <c r="G148" s="9">
         <v>0</v>
@@ -29023,11 +29025,11 @@
         <v>125</v>
       </c>
       <c r="I148" s="8" t="s">
-        <v>1563</v>
+        <v>1560</v>
       </c>
       <c r="K148" s="5" t="str">
-        <f t="shared" ref="K148" si="17">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B148&amp;"'"&amp;","&amp;E148&amp;","&amp;"'"&amp;C148&amp;"'"&amp;","&amp;"'"&amp;D148&amp;"'"&amp;","&amp;"'"&amp;F148&amp;"'"&amp;","&amp;G148&amp;","&amp;H148&amp;","&amp;"'"&amp;I148&amp;"'"&amp;");"</f>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',34,'Meranti','','メランティ',0,0.0,'中域寄りで温かめ、マホガニー系に近い。');</v>
+        <f t="shared" si="16"/>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',33,'Okoume','','オクメ',0,0.0,'マホガニーに近く、中低域が豊かで軽量。');</v>
       </c>
     </row>
     <row r="149" spans="2:11">
@@ -29035,14 +29037,14 @@
         <v>1778</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>1564</v>
+        <v>1562</v>
       </c>
       <c r="D149" s="8"/>
       <c r="E149" s="8">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F149" s="8" t="s">
-        <v>1565</v>
+        <v>1561</v>
       </c>
       <c r="G149" s="9">
         <v>0</v>
@@ -29051,11 +29053,11 @@
         <v>125</v>
       </c>
       <c r="I149" s="8" t="s">
-        <v>1569</v>
+        <v>1563</v>
       </c>
       <c r="K149" s="5" t="str">
-        <f t="shared" ref="K149" si="18">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B149&amp;"'"&amp;","&amp;E149&amp;","&amp;"'"&amp;C149&amp;"'"&amp;","&amp;"'"&amp;D149&amp;"'"&amp;","&amp;"'"&amp;F149&amp;"'"&amp;","&amp;G149&amp;","&amp;H149&amp;","&amp;"'"&amp;I149&amp;"'"&amp;");"</f>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',35,'Sakura','','サクラ',0,0.0,'中高域が明るく立ち上がりが速い、日本らしい軽快で抜けの良いサウンド。');</v>
+        <f t="shared" ref="K149" si="17">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B149&amp;"'"&amp;","&amp;E149&amp;","&amp;"'"&amp;C149&amp;"'"&amp;","&amp;"'"&amp;D149&amp;"'"&amp;","&amp;"'"&amp;F149&amp;"'"&amp;","&amp;G149&amp;","&amp;H149&amp;","&amp;"'"&amp;I149&amp;"'"&amp;");"</f>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',34,'Meranti','','メランティ',0,0.0,'中域寄りで温かめ、マホガニー系に近い。');</v>
       </c>
     </row>
     <row r="150" spans="2:11">
@@ -29063,14 +29065,14 @@
         <v>1778</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>1566</v>
+        <v>1564</v>
       </c>
       <c r="D150" s="8"/>
       <c r="E150" s="8">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F150" s="8" t="s">
-        <v>1567</v>
+        <v>1565</v>
       </c>
       <c r="G150" s="9">
         <v>0</v>
@@ -29079,11 +29081,11 @@
         <v>125</v>
       </c>
       <c r="I150" s="8" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
       <c r="K150" s="5" t="str">
-        <f t="shared" si="16"/>
-        <v>INSERT INTO m_code VALUES ('guitar_woods',36,'Tochi','','トチ',0,0.0,'メイプルに近いクリアさと華やかさを持ちつつ、やや柔らかく豊かな倍音.');</v>
+        <f t="shared" ref="K150" si="18">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B150&amp;"'"&amp;","&amp;E150&amp;","&amp;"'"&amp;C150&amp;"'"&amp;","&amp;"'"&amp;D150&amp;"'"&amp;","&amp;"'"&amp;F150&amp;"'"&amp;","&amp;G150&amp;","&amp;H150&amp;","&amp;"'"&amp;I150&amp;"'"&amp;");"</f>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',35,'Sakura','','サクラ',0,0.0,'中高域が明るく立ち上がりが速い、日本らしい軽快で抜けの良いサウンド。');</v>
       </c>
     </row>
     <row r="151" spans="2:11">
@@ -29091,14 +29093,14 @@
         <v>1778</v>
       </c>
       <c r="C151" s="8" t="s">
-        <v>1424</v>
+        <v>1566</v>
       </c>
       <c r="D151" s="8"/>
       <c r="E151" s="8">
-        <v>99</v>
+        <v>36</v>
       </c>
       <c r="F151" s="8" t="s">
-        <v>1423</v>
+        <v>1567</v>
       </c>
       <c r="G151" s="9">
         <v>0</v>
@@ -29106,62 +29108,64 @@
       <c r="H151" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="I151" s="8"/>
+      <c r="I151" s="8" t="s">
+        <v>1568</v>
+      </c>
       <c r="K151" s="5" t="str">
-        <f>"INSERT INTO m_code VALUES ("&amp;"'"&amp;B151&amp;"'"&amp;","&amp;E151&amp;","&amp;"'"&amp;C151&amp;"'"&amp;","&amp;"'"&amp;D151&amp;"'"&amp;","&amp;"'"&amp;F151&amp;"'"&amp;","&amp;G151&amp;","&amp;H151&amp;","&amp;"'"&amp;I151&amp;"'"&amp;");"</f>
+        <f t="shared" si="16"/>
+        <v>INSERT INTO m_code VALUES ('guitar_woods',36,'Tochi','','トチ',0,0.0,'メイプルに近いクリアさと華やかさを持ちつつ、やや柔らかく豊かな倍音.');</v>
+      </c>
+    </row>
+    <row r="152" spans="2:11">
+      <c r="B152" s="8" t="s">
+        <v>1778</v>
+      </c>
+      <c r="C152" s="8" t="s">
+        <v>1424</v>
+      </c>
+      <c r="D152" s="8"/>
+      <c r="E152" s="8">
+        <v>99</v>
+      </c>
+      <c r="F152" s="8" t="s">
+        <v>1423</v>
+      </c>
+      <c r="G152" s="9">
+        <v>0</v>
+      </c>
+      <c r="H152" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="I152" s="8"/>
+      <c r="K152" s="5" t="str">
+        <f>"INSERT INTO m_code VALUES ("&amp;"'"&amp;B152&amp;"'"&amp;","&amp;E152&amp;","&amp;"'"&amp;C152&amp;"'"&amp;","&amp;"'"&amp;D152&amp;"'"&amp;","&amp;"'"&amp;F152&amp;"'"&amp;","&amp;G152&amp;","&amp;H152&amp;","&amp;"'"&amp;I152&amp;"'"&amp;");"</f>
         <v>INSERT INTO m_code VALUES ('guitar_woods',99,'Unknown','','？？',0,0.0,'');</v>
       </c>
     </row>
-    <row r="152" spans="2:11">
-      <c r="B152" s="6" t="s">
+    <row r="153" spans="2:11">
+      <c r="B153" s="6" t="s">
         <v>1503</v>
       </c>
-      <c r="C152" s="6" t="s">
+      <c r="C153" s="6" t="s">
         <v>1502</v>
       </c>
-      <c r="D152" s="6" t="s">
+      <c r="D153" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="E152" s="7" t="s">
+      <c r="E153" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="F152" s="6" t="s">
+      <c r="F153" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="G152" s="6" t="s">
+      <c r="G153" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="H152" s="6" t="s">
+      <c r="H153" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="I152" s="6" t="s">
+      <c r="I153" s="6" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="153" spans="2:11">
-      <c r="B153" s="8" t="s">
-        <v>1779</v>
-      </c>
-      <c r="C153" s="8" t="s">
-        <v>1504</v>
-      </c>
-      <c r="D153" s="8"/>
-      <c r="E153" s="8">
-        <v>1</v>
-      </c>
-      <c r="F153" s="8" t="s">
-        <v>1520</v>
-      </c>
-      <c r="G153" s="9">
-        <v>0</v>
-      </c>
-      <c r="H153" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="I153" s="8"/>
-      <c r="K153" s="5" t="str">
-        <f t="shared" ref="K153:K175" si="19">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B153&amp;"'"&amp;","&amp;E153&amp;","&amp;"'"&amp;C153&amp;"'"&amp;","&amp;"'"&amp;D153&amp;"'"&amp;","&amp;"'"&amp;F153&amp;"'"&amp;","&amp;G153&amp;","&amp;H153&amp;","&amp;"'"&amp;I153&amp;"'"&amp;");"</f>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',1,'Red','','レッド',0,0.0,'');</v>
       </c>
     </row>
     <row r="154" spans="2:11">
@@ -29169,14 +29173,14 @@
         <v>1779</v>
       </c>
       <c r="C154" s="8" t="s">
-        <v>1518</v>
+        <v>1504</v>
       </c>
       <c r="D154" s="8"/>
       <c r="E154" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F154" s="8" t="s">
-        <v>1521</v>
+        <v>1520</v>
       </c>
       <c r="G154" s="9">
         <v>0</v>
@@ -29186,8 +29190,8 @@
       </c>
       <c r="I154" s="8"/>
       <c r="K154" s="5" t="str">
-        <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',2,'Pink','','ピンク',0,0.0,'');</v>
+        <f t="shared" ref="K154:K176" si="19">"INSERT INTO m_code VALUES ("&amp;"'"&amp;B154&amp;"'"&amp;","&amp;E154&amp;","&amp;"'"&amp;C154&amp;"'"&amp;","&amp;"'"&amp;D154&amp;"'"&amp;","&amp;"'"&amp;F154&amp;"'"&amp;","&amp;G154&amp;","&amp;H154&amp;","&amp;"'"&amp;I154&amp;"'"&amp;");"</f>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',1,'Red','','レッド',0,0.0,'');</v>
       </c>
     </row>
     <row r="155" spans="2:11">
@@ -29195,14 +29199,14 @@
         <v>1779</v>
       </c>
       <c r="C155" s="8" t="s">
-        <v>1505</v>
+        <v>1518</v>
       </c>
       <c r="D155" s="8"/>
       <c r="E155" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F155" s="8" t="s">
-        <v>1522</v>
+        <v>1521</v>
       </c>
       <c r="G155" s="9">
         <v>0</v>
@@ -29213,7 +29217,7 @@
       <c r="I155" s="8"/>
       <c r="K155" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',3,'Orange','','オレンジ',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',2,'Pink','','ピンク',0,0.0,'');</v>
       </c>
     </row>
     <row r="156" spans="2:11">
@@ -29221,14 +29225,14 @@
         <v>1779</v>
       </c>
       <c r="C156" s="8" t="s">
-        <v>1506</v>
+        <v>1505</v>
       </c>
       <c r="D156" s="8"/>
       <c r="E156" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F156" s="8" t="s">
-        <v>1523</v>
+        <v>1522</v>
       </c>
       <c r="G156" s="9">
         <v>0</v>
@@ -29239,7 +29243,7 @@
       <c r="I156" s="8"/>
       <c r="K156" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',4,'Yellow','','イエロー',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',3,'Orange','','オレンジ',0,0.0,'');</v>
       </c>
     </row>
     <row r="157" spans="2:11">
@@ -29247,14 +29251,14 @@
         <v>1779</v>
       </c>
       <c r="C157" s="8" t="s">
-        <v>1507</v>
+        <v>1506</v>
       </c>
       <c r="D157" s="8"/>
       <c r="E157" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F157" s="8" t="s">
-        <v>1524</v>
+        <v>1523</v>
       </c>
       <c r="G157" s="9">
         <v>0</v>
@@ -29265,7 +29269,7 @@
       <c r="I157" s="8"/>
       <c r="K157" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',5,'Green','','グリーン',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',4,'Yellow','','イエロー',0,0.0,'');</v>
       </c>
     </row>
     <row r="158" spans="2:11">
@@ -29273,14 +29277,14 @@
         <v>1779</v>
       </c>
       <c r="C158" s="8" t="s">
-        <v>1508</v>
+        <v>1507</v>
       </c>
       <c r="D158" s="8"/>
       <c r="E158" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F158" s="8" t="s">
-        <v>1525</v>
+        <v>1524</v>
       </c>
       <c r="G158" s="9">
         <v>0</v>
@@ -29291,7 +29295,7 @@
       <c r="I158" s="8"/>
       <c r="K158" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',6,'SkyBlue','','スカイブルー',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',5,'Green','','グリーン',0,0.0,'');</v>
       </c>
     </row>
     <row r="159" spans="2:11">
@@ -29299,14 +29303,14 @@
         <v>1779</v>
       </c>
       <c r="C159" s="8" t="s">
-        <v>1509</v>
+        <v>1508</v>
       </c>
       <c r="D159" s="8"/>
       <c r="E159" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F159" s="8" t="s">
-        <v>1526</v>
+        <v>1525</v>
       </c>
       <c r="G159" s="9">
         <v>0</v>
@@ -29317,7 +29321,7 @@
       <c r="I159" s="8"/>
       <c r="K159" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',7,'Blue','','ブルー',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',6,'SkyBlue','','スカイブルー',0,0.0,'');</v>
       </c>
     </row>
     <row r="160" spans="2:11">
@@ -29325,14 +29329,14 @@
         <v>1779</v>
       </c>
       <c r="C160" s="8" t="s">
-        <v>1510</v>
+        <v>1509</v>
       </c>
       <c r="D160" s="8"/>
       <c r="E160" s="8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F160" s="8" t="s">
-        <v>1527</v>
+        <v>1526</v>
       </c>
       <c r="G160" s="9">
         <v>0</v>
@@ -29343,7 +29347,7 @@
       <c r="I160" s="8"/>
       <c r="K160" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',8,'Purple','','パープル',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',7,'Blue','','ブルー',0,0.0,'');</v>
       </c>
     </row>
     <row r="161" spans="2:11">
@@ -29351,14 +29355,14 @@
         <v>1779</v>
       </c>
       <c r="C161" s="8" t="s">
-        <v>1511</v>
+        <v>1510</v>
       </c>
       <c r="D161" s="8"/>
       <c r="E161" s="8">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F161" s="8" t="s">
-        <v>1528</v>
+        <v>1527</v>
       </c>
       <c r="G161" s="9">
         <v>0</v>
@@ -29369,7 +29373,7 @@
       <c r="I161" s="8"/>
       <c r="K161" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',9,'Gray','','グレー',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',8,'Purple','','パープル',0,0.0,'');</v>
       </c>
     </row>
     <row r="162" spans="2:11">
@@ -29377,14 +29381,14 @@
         <v>1779</v>
       </c>
       <c r="C162" s="8" t="s">
-        <v>1512</v>
+        <v>1511</v>
       </c>
       <c r="D162" s="8"/>
       <c r="E162" s="8">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F162" s="8" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="G162" s="9">
         <v>0</v>
@@ -29395,7 +29399,7 @@
       <c r="I162" s="8"/>
       <c r="K162" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',10,'Black','','ブラック',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',9,'Gray','','グレー',0,0.0,'');</v>
       </c>
     </row>
     <row r="163" spans="2:11">
@@ -29403,14 +29407,14 @@
         <v>1779</v>
       </c>
       <c r="C163" s="8" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="D163" s="8"/>
       <c r="E163" s="8">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F163" s="8" t="s">
-        <v>1530</v>
+        <v>1529</v>
       </c>
       <c r="G163" s="9">
         <v>0</v>
@@ -29421,7 +29425,7 @@
       <c r="I163" s="8"/>
       <c r="K163" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',11,'White','','ホワイト',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',10,'Black','','ブラック',0,0.0,'');</v>
       </c>
     </row>
     <row r="164" spans="2:11">
@@ -29429,14 +29433,14 @@
         <v>1779</v>
       </c>
       <c r="C164" s="8" t="s">
-        <v>1514</v>
+        <v>1513</v>
       </c>
       <c r="D164" s="8"/>
       <c r="E164" s="8">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F164" s="8" t="s">
-        <v>1531</v>
+        <v>1530</v>
       </c>
       <c r="G164" s="9">
         <v>0</v>
@@ -29447,7 +29451,7 @@
       <c r="I164" s="8"/>
       <c r="K164" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',12,'Natural','','ナチュラル',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',11,'White','','ホワイト',0,0.0,'');</v>
       </c>
     </row>
     <row r="165" spans="2:11">
@@ -29455,14 +29459,14 @@
         <v>1779</v>
       </c>
       <c r="C165" s="8" t="s">
-        <v>1519</v>
+        <v>1514</v>
       </c>
       <c r="D165" s="8"/>
       <c r="E165" s="8">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F165" s="8" t="s">
-        <v>1532</v>
+        <v>1531</v>
       </c>
       <c r="G165" s="9">
         <v>0</v>
@@ -29473,7 +29477,7 @@
       <c r="I165" s="8"/>
       <c r="K165" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',13,'Brown','','ブラウン',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',12,'Natural','','ナチュラル',0,0.0,'');</v>
       </c>
     </row>
     <row r="166" spans="2:11">
@@ -29481,14 +29485,14 @@
         <v>1779</v>
       </c>
       <c r="C166" s="8" t="s">
-        <v>1515</v>
+        <v>1519</v>
       </c>
       <c r="D166" s="8"/>
       <c r="E166" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F166" s="8" t="s">
-        <v>1533</v>
+        <v>1532</v>
       </c>
       <c r="G166" s="9">
         <v>0</v>
@@ -29499,7 +29503,7 @@
       <c r="I166" s="8"/>
       <c r="K166" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',14,'Gold','','ゴールド',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',13,'Brown','','ブラウン',0,0.0,'');</v>
       </c>
     </row>
     <row r="167" spans="2:11">
@@ -29507,14 +29511,14 @@
         <v>1779</v>
       </c>
       <c r="C167" s="8" t="s">
-        <v>1516</v>
+        <v>1515</v>
       </c>
       <c r="D167" s="8"/>
       <c r="E167" s="8">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F167" s="8" t="s">
-        <v>1534</v>
+        <v>1533</v>
       </c>
       <c r="G167" s="9">
         <v>0</v>
@@ -29525,7 +29529,7 @@
       <c r="I167" s="8"/>
       <c r="K167" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('guitar_colors',15,'Silver','','シルバー',0,0.0,'');</v>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',14,'Gold','','ゴールド',0,0.0,'');</v>
       </c>
     </row>
     <row r="168" spans="2:11">
@@ -29533,14 +29537,14 @@
         <v>1779</v>
       </c>
       <c r="C168" s="8" t="s">
-        <v>1517</v>
+        <v>1516</v>
       </c>
       <c r="D168" s="8"/>
       <c r="E168" s="8">
-        <v>99</v>
+        <v>15</v>
       </c>
       <c r="F168" s="8" t="s">
-        <v>1535</v>
+        <v>1534</v>
       </c>
       <c r="G168" s="9">
         <v>0</v>
@@ -29551,59 +29555,59 @@
       <c r="I168" s="8"/>
       <c r="K168" s="5" t="str">
         <f t="shared" si="19"/>
+        <v>INSERT INTO m_code VALUES ('guitar_colors',15,'Silver','','シルバー',0,0.0,'');</v>
+      </c>
+    </row>
+    <row r="169" spans="2:11">
+      <c r="B169" s="8" t="s">
+        <v>1779</v>
+      </c>
+      <c r="C169" s="8" t="s">
+        <v>1517</v>
+      </c>
+      <c r="D169" s="8"/>
+      <c r="E169" s="8">
+        <v>99</v>
+      </c>
+      <c r="F169" s="8" t="s">
+        <v>1535</v>
+      </c>
+      <c r="G169" s="9">
+        <v>0</v>
+      </c>
+      <c r="H169" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="I169" s="8"/>
+      <c r="K169" s="5" t="str">
+        <f t="shared" si="19"/>
         <v>INSERT INTO m_code VALUES ('guitar_colors',99,'Others','','その他',0,0.0,'');</v>
       </c>
     </row>
-    <row r="169" spans="2:11">
-      <c r="B169" s="6" t="s">
+    <row r="170" spans="2:11">
+      <c r="B170" s="6" t="s">
         <v>1888</v>
       </c>
-      <c r="C169" s="6" t="s">
+      <c r="C170" s="6" t="s">
         <v>1889</v>
       </c>
-      <c r="D169" s="6" t="s">
+      <c r="D170" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="E169" s="7" t="s">
+      <c r="E170" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="F169" s="6" t="s">
+      <c r="F170" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="G169" s="6" t="s">
+      <c r="G170" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="H169" s="6" t="s">
+      <c r="H170" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="I169" s="6" t="s">
+      <c r="I170" s="6" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="170" spans="2:11">
-      <c r="B170" s="8" t="s">
-        <v>1892</v>
-      </c>
-      <c r="C170" s="8" t="s">
-        <v>1890</v>
-      </c>
-      <c r="D170" s="8"/>
-      <c r="E170" s="8">
-        <v>1</v>
-      </c>
-      <c r="F170" s="8"/>
-      <c r="G170" s="9">
-        <v>0</v>
-      </c>
-      <c r="H170" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="I170" s="8" t="s">
-        <v>1893</v>
-      </c>
-      <c r="K170" s="5" t="str">
-        <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('batch_status',1,'SUCCESS','','',0,0.0,'処理成功');</v>
       </c>
     </row>
     <row r="171" spans="2:11">
@@ -29611,11 +29615,11 @@
         <v>1892</v>
       </c>
       <c r="C171" s="8" t="s">
-        <v>1891</v>
+        <v>1890</v>
       </c>
       <c r="D171" s="8"/>
       <c r="E171" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F171" s="8"/>
       <c r="G171" s="9">
@@ -29625,11 +29629,11 @@
         <v>125</v>
       </c>
       <c r="I171" s="8" t="s">
-        <v>1894</v>
+        <v>1893</v>
       </c>
       <c r="K171" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('batch_status',2,'STARTED','','',0,0.0,'処理開始。いずかのステータスに遷移する。');</v>
+        <v>INSERT INTO m_code VALUES ('batch_status',1,'SUCCESS','','',0,0.0,'処理成功');</v>
       </c>
     </row>
     <row r="172" spans="2:11">
@@ -29637,11 +29641,11 @@
         <v>1892</v>
       </c>
       <c r="C172" s="8" t="s">
-        <v>1881</v>
+        <v>1891</v>
       </c>
       <c r="D172" s="8"/>
       <c r="E172" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F172" s="8"/>
       <c r="G172" s="9">
@@ -29651,11 +29655,11 @@
         <v>125</v>
       </c>
       <c r="I172" s="8" t="s">
-        <v>1895</v>
+        <v>1894</v>
       </c>
       <c r="K172" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('batch_status',3,'NOT_STARTED','','',0,0.0,'予定時刻に開始されていない。');</v>
+        <v>INSERT INTO m_code VALUES ('batch_status',2,'STARTED','','',0,0.0,'処理開始。いずかのステータスに遷移する。');</v>
       </c>
     </row>
     <row r="173" spans="2:11">
@@ -29663,11 +29667,11 @@
         <v>1892</v>
       </c>
       <c r="C173" s="8" t="s">
-        <v>1879</v>
+        <v>1881</v>
       </c>
       <c r="D173" s="8"/>
       <c r="E173" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F173" s="8"/>
       <c r="G173" s="9">
@@ -29677,11 +29681,11 @@
         <v>125</v>
       </c>
       <c r="I173" s="8" t="s">
-        <v>1896</v>
+        <v>1895</v>
       </c>
       <c r="K173" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('batch_status',4,'ERROR','','',0,0.0,'例外、パニック等が発生した。');</v>
+        <v>INSERT INTO m_code VALUES ('batch_status',3,'NOT_STARTED','','',0,0.0,'予定時刻に開始されていない。');</v>
       </c>
     </row>
     <row r="174" spans="2:11">
@@ -29689,11 +29693,11 @@
         <v>1892</v>
       </c>
       <c r="C174" s="8" t="s">
-        <v>1882</v>
+        <v>1879</v>
       </c>
       <c r="D174" s="8"/>
       <c r="E174" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F174" s="8"/>
       <c r="G174" s="9">
@@ -29703,11 +29707,11 @@
         <v>125</v>
       </c>
       <c r="I174" s="8" t="s">
-        <v>1898</v>
+        <v>1896</v>
       </c>
       <c r="K174" s="5" t="str">
         <f t="shared" si="19"/>
-        <v>INSERT INTO m_code VALUES ('batch_status',5,'SLOW','','',0,0.0,'想定時間内に処理が終了しなかった。');</v>
+        <v>INSERT INTO m_code VALUES ('batch_status',4,'ERROR','','',0,0.0,'例外、パニック等が発生した。');</v>
       </c>
     </row>
     <row r="175" spans="2:11">
@@ -29715,11 +29719,11 @@
         <v>1892</v>
       </c>
       <c r="C175" s="8" t="s">
-        <v>1880</v>
+        <v>1882</v>
       </c>
       <c r="D175" s="8"/>
       <c r="E175" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F175" s="8"/>
       <c r="G175" s="9">
@@ -29729,9 +29733,35 @@
         <v>125</v>
       </c>
       <c r="I175" s="8" t="s">
+        <v>1898</v>
+      </c>
+      <c r="K175" s="5" t="str">
+        <f t="shared" si="19"/>
+        <v>INSERT INTO m_code VALUES ('batch_status',5,'SLOW','','',0,0.0,'想定時間内に処理が終了しなかった。');</v>
+      </c>
+    </row>
+    <row r="176" spans="2:11">
+      <c r="B176" s="8" t="s">
+        <v>1892</v>
+      </c>
+      <c r="C176" s="8" t="s">
+        <v>1880</v>
+      </c>
+      <c r="D176" s="8"/>
+      <c r="E176" s="8">
+        <v>6</v>
+      </c>
+      <c r="F176" s="8"/>
+      <c r="G176" s="9">
+        <v>0</v>
+      </c>
+      <c r="H176" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="I176" s="8" t="s">
         <v>1897</v>
       </c>
-      <c r="K175" s="5" t="str">
+      <c r="K176" s="5" t="str">
         <f t="shared" si="19"/>
         <v>INSERT INTO m_code VALUES ('batch_status',6,'TIMEOUT','','',0,0.0,'時間内に処理が終了しなかった。');</v>
       </c>
@@ -29745,10 +29775,10 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F51B408-D4E3-46FE-97DE-15AB67B6AAB6}">
   <dimension ref="B1:Q100"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="1" width="9" style="5"/>
-    <col min="2" max="2" width="12.75" style="5" customWidth="1"/>
+    <col min="2" max="2" width="12.69921875" style="5" customWidth="1"/>
     <col min="3" max="3" width="17.5" style="5" customWidth="1"/>
     <col min="4" max="16384" width="9" style="5"/>
   </cols>
@@ -29859,7 +29889,7 @@
         <v>150</v>
       </c>
       <c r="L6" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B6&amp;"'"&amp;","&amp;"'"&amp;C6&amp;"'"&amp;","&amp;VLOOKUP(D6,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E6&amp;","&amp;F6&amp;","&amp;G6&amp;","&amp;H6&amp;","&amp;VLOOKUP(I6,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B6&amp;"'"&amp;","&amp;"'"&amp;C6&amp;"'"&amp;","&amp;VLOOKUP(D6,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E6&amp;","&amp;F6&amp;","&amp;G6&amp;","&amp;H6&amp;","&amp;VLOOKUP(I6,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster001','キラービー',1,110,12,16,0.3,1);</v>
       </c>
     </row>
@@ -29892,7 +29922,7 @@
         <v>150</v>
       </c>
       <c r="L7" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B7&amp;"'"&amp;","&amp;"'"&amp;C7&amp;"'"&amp;","&amp;VLOOKUP(D7,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E7&amp;","&amp;F7&amp;","&amp;G7&amp;","&amp;H7&amp;","&amp;VLOOKUP(I7,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B7&amp;"'"&amp;","&amp;"'"&amp;C7&amp;"'"&amp;","&amp;VLOOKUP(D7,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E7&amp;","&amp;F7&amp;","&amp;G7&amp;","&amp;H7&amp;","&amp;VLOOKUP(I7,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster002','アサシンバグ',1,132,15,20,0.3,1);</v>
       </c>
     </row>
@@ -29925,7 +29955,7 @@
         <v>150</v>
       </c>
       <c r="L8" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B8&amp;"'"&amp;","&amp;"'"&amp;C8&amp;"'"&amp;","&amp;VLOOKUP(D8,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E8&amp;","&amp;F8&amp;","&amp;G8&amp;","&amp;H8&amp;","&amp;VLOOKUP(I8,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B8&amp;"'"&amp;","&amp;"'"&amp;C8&amp;"'"&amp;","&amp;VLOOKUP(D8,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E8&amp;","&amp;F8&amp;","&amp;G8&amp;","&amp;H8&amp;","&amp;VLOOKUP(I8,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster003','ラスターバグ',1,158,19,26,0.3,1);</v>
       </c>
     </row>
@@ -29955,7 +29985,7 @@
         <v>34</v>
       </c>
       <c r="L9" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B9&amp;"'"&amp;","&amp;"'"&amp;C9&amp;"'"&amp;","&amp;VLOOKUP(D9,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E9&amp;","&amp;F9&amp;","&amp;G9&amp;","&amp;H9&amp;","&amp;VLOOKUP(I9,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B9&amp;"'"&amp;","&amp;"'"&amp;C9&amp;"'"&amp;","&amp;VLOOKUP(D9,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E9&amp;","&amp;F9&amp;","&amp;G9&amp;","&amp;H9&amp;","&amp;VLOOKUP(I9,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster004','カーミラ',2,100,10,13,0.13,2);</v>
       </c>
     </row>
@@ -29988,7 +30018,7 @@
         <v>34</v>
       </c>
       <c r="L10" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B10&amp;"'"&amp;","&amp;"'"&amp;C10&amp;"'"&amp;","&amp;VLOOKUP(D10,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E10&amp;","&amp;F10&amp;","&amp;G10&amp;","&amp;H10&amp;","&amp;VLOOKUP(I10,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B10&amp;"'"&amp;","&amp;"'"&amp;C10&amp;"'"&amp;","&amp;VLOOKUP(D10,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E10&amp;","&amp;F10&amp;","&amp;G10&amp;","&amp;H10&amp;","&amp;VLOOKUP(I10,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster005','カーミラクイーン',2,120,13,16,0.15,2);</v>
       </c>
     </row>
@@ -30018,7 +30048,7 @@
         <v>36</v>
       </c>
       <c r="L11" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B11&amp;"'"&amp;","&amp;"'"&amp;C11&amp;"'"&amp;","&amp;VLOOKUP(D11,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E11&amp;","&amp;F11&amp;","&amp;G11&amp;","&amp;H11&amp;","&amp;VLOOKUP(I11,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B11&amp;"'"&amp;","&amp;"'"&amp;C11&amp;"'"&amp;","&amp;VLOOKUP(D11,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E11&amp;","&amp;F11&amp;","&amp;G11&amp;","&amp;H11&amp;","&amp;VLOOKUP(I11,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster006','デーモン',3,130,15,7,0.08,5);</v>
       </c>
     </row>
@@ -30051,7 +30081,7 @@
         <v>36</v>
       </c>
       <c r="L12" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B12&amp;"'"&amp;","&amp;"'"&amp;C12&amp;"'"&amp;","&amp;VLOOKUP(D12,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E12&amp;","&amp;F12&amp;","&amp;G12&amp;","&amp;H12&amp;","&amp;VLOOKUP(I12,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B12&amp;"'"&amp;","&amp;"'"&amp;C12&amp;"'"&amp;","&amp;VLOOKUP(D12,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E12&amp;","&amp;F12&amp;","&amp;G12&amp;","&amp;H12&amp;","&amp;VLOOKUP(I12,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster007','グレートデーモン',3,156,19,9,0.1,5);</v>
       </c>
     </row>
@@ -30081,7 +30111,7 @@
         <v>35</v>
       </c>
       <c r="L13" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B13&amp;"'"&amp;","&amp;"'"&amp;C13&amp;"'"&amp;","&amp;VLOOKUP(D13,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E13&amp;","&amp;F13&amp;","&amp;G13&amp;","&amp;H13&amp;","&amp;VLOOKUP(I13,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B13&amp;"'"&amp;","&amp;"'"&amp;C13&amp;"'"&amp;","&amp;VLOOKUP(D13,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E13&amp;","&amp;F13&amp;","&amp;G13&amp;","&amp;H13&amp;","&amp;VLOOKUP(I13,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster008','ゴブリン',4,120,11,10,0.15,4);</v>
       </c>
     </row>
@@ -30114,7 +30144,7 @@
         <v>35</v>
       </c>
       <c r="L14" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B14&amp;"'"&amp;","&amp;"'"&amp;C14&amp;"'"&amp;","&amp;VLOOKUP(D14,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E14&amp;","&amp;F14&amp;","&amp;G14&amp;","&amp;H14&amp;","&amp;VLOOKUP(I14,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B14&amp;"'"&amp;","&amp;"'"&amp;C14&amp;"'"&amp;","&amp;VLOOKUP(D14,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E14&amp;","&amp;F14&amp;","&amp;G14&amp;","&amp;H14&amp;","&amp;VLOOKUP(I14,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster009','ゴブリンガード',4,144,14,13,0.15,4);</v>
       </c>
     </row>
@@ -30147,7 +30177,7 @@
         <v>35</v>
       </c>
       <c r="L15" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B15&amp;"'"&amp;","&amp;"'"&amp;C15&amp;"'"&amp;","&amp;VLOOKUP(D15,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E15&amp;","&amp;F15&amp;","&amp;G15&amp;","&amp;H15&amp;","&amp;VLOOKUP(I15,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B15&amp;"'"&amp;","&amp;"'"&amp;C15&amp;"'"&amp;","&amp;VLOOKUP(D15,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E15&amp;","&amp;F15&amp;","&amp;G15&amp;","&amp;H15&amp;","&amp;VLOOKUP(I15,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster010','ゴブリンロード',4,172,18,16,0.15,4);</v>
       </c>
     </row>
@@ -30177,7 +30207,7 @@
         <v>151</v>
       </c>
       <c r="L16" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B16&amp;"'"&amp;","&amp;"'"&amp;C16&amp;"'"&amp;","&amp;VLOOKUP(D16,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E16&amp;","&amp;F16&amp;","&amp;G16&amp;","&amp;H16&amp;","&amp;VLOOKUP(I16,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B16&amp;"'"&amp;","&amp;"'"&amp;C16&amp;"'"&amp;","&amp;VLOOKUP(D16,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E16&amp;","&amp;F16&amp;","&amp;G16&amp;","&amp;H16&amp;","&amp;VLOOKUP(I16,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster011','マシンゴーレム',5,140,17,5,0.02,3);</v>
       </c>
     </row>
@@ -30210,7 +30240,7 @@
         <v>151</v>
       </c>
       <c r="L17" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B17&amp;"'"&amp;","&amp;"'"&amp;C17&amp;"'"&amp;","&amp;VLOOKUP(D17,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E17&amp;","&amp;F17&amp;","&amp;G17&amp;","&amp;H17&amp;","&amp;VLOOKUP(I17,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B17&amp;"'"&amp;","&amp;"'"&amp;C17&amp;"'"&amp;","&amp;VLOOKUP(D17,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E17&amp;","&amp;F17&amp;","&amp;G17&amp;","&amp;H17&amp;","&amp;VLOOKUP(I17,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster012','ガーディアン',5,168,22,6,0.04,3);</v>
       </c>
     </row>
@@ -30243,7 +30273,7 @@
         <v>151</v>
       </c>
       <c r="L18" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B18&amp;"'"&amp;","&amp;"'"&amp;C18&amp;"'"&amp;","&amp;VLOOKUP(D18,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E18&amp;","&amp;F18&amp;","&amp;G18&amp;","&amp;H18&amp;","&amp;VLOOKUP(I18,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B18&amp;"'"&amp;","&amp;"'"&amp;C18&amp;"'"&amp;","&amp;VLOOKUP(D18,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E18&amp;","&amp;F18&amp;","&amp;G18&amp;","&amp;H18&amp;","&amp;VLOOKUP(I18,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster013','デスマシン',5,201,28,7,0.05,3);</v>
       </c>
     </row>
@@ -30273,7 +30303,7 @@
         <v>35</v>
       </c>
       <c r="L19" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B19&amp;"'"&amp;","&amp;"'"&amp;C19&amp;"'"&amp;","&amp;VLOOKUP(D19,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E19&amp;","&amp;F19&amp;","&amp;G19&amp;","&amp;H19&amp;","&amp;VLOOKUP(I19,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B19&amp;"'"&amp;","&amp;"'"&amp;C19&amp;"'"&amp;","&amp;VLOOKUP(D19,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E19&amp;","&amp;F19&amp;","&amp;G19&amp;","&amp;H19&amp;","&amp;VLOOKUP(I19,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster014','ハーピー',6,100,8,14,0.2,4);</v>
       </c>
     </row>
@@ -30306,7 +30336,7 @@
         <v>35</v>
       </c>
       <c r="L20" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B20&amp;"'"&amp;","&amp;"'"&amp;C20&amp;"'"&amp;","&amp;VLOOKUP(D20,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E20&amp;","&amp;F20&amp;","&amp;G20&amp;","&amp;H20&amp;","&amp;VLOOKUP(I20,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B20&amp;"'"&amp;","&amp;"'"&amp;C20&amp;"'"&amp;","&amp;VLOOKUP(D20,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E20&amp;","&amp;F20&amp;","&amp;G20&amp;","&amp;H20&amp;","&amp;VLOOKUP(I20,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster015','セイレーン',6,120,10,18,0.23,4);</v>
       </c>
     </row>
@@ -30336,7 +30366,7 @@
         <v>34</v>
       </c>
       <c r="L21" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B21&amp;"'"&amp;","&amp;"'"&amp;C21&amp;"'"&amp;","&amp;VLOOKUP(D21,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E21&amp;","&amp;F21&amp;","&amp;G21&amp;","&amp;H21&amp;","&amp;VLOOKUP(I21,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B21&amp;"'"&amp;","&amp;"'"&amp;C21&amp;"'"&amp;","&amp;VLOOKUP(D21,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E21&amp;","&amp;F21&amp;","&amp;G21&amp;","&amp;H21&amp;","&amp;VLOOKUP(I21,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster016','アーマーナイト',7,120,13,8,0.05,2);</v>
       </c>
     </row>
@@ -30369,7 +30399,7 @@
         <v>34</v>
       </c>
       <c r="L22" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B22&amp;"'"&amp;","&amp;"'"&amp;C22&amp;"'"&amp;","&amp;VLOOKUP(D22,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E22&amp;","&amp;F22&amp;","&amp;G22&amp;","&amp;H22&amp;","&amp;VLOOKUP(I22,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B22&amp;"'"&amp;","&amp;"'"&amp;C22&amp;"'"&amp;","&amp;VLOOKUP(D22,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E22&amp;","&amp;F22&amp;","&amp;G22&amp;","&amp;H22&amp;","&amp;VLOOKUP(I22,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster017','ダークナイト',7,144,16,10,0.05,2);</v>
       </c>
     </row>
@@ -30402,7 +30432,7 @@
         <v>34</v>
       </c>
       <c r="L23" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B23&amp;"'"&amp;","&amp;"'"&amp;C23&amp;"'"&amp;","&amp;VLOOKUP(D23,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E23&amp;","&amp;F23&amp;","&amp;G23&amp;","&amp;H23&amp;","&amp;VLOOKUP(I23,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B23&amp;"'"&amp;","&amp;"'"&amp;C23&amp;"'"&amp;","&amp;VLOOKUP(D23,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E23&amp;","&amp;F23&amp;","&amp;G23&amp;","&amp;H23&amp;","&amp;VLOOKUP(I23,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster018','ターミネータ',7,172,20,13,0.07,2);</v>
       </c>
     </row>
@@ -30432,7 +30462,7 @@
         <v>35</v>
       </c>
       <c r="L24" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B24&amp;"'"&amp;","&amp;"'"&amp;C24&amp;"'"&amp;","&amp;VLOOKUP(D24,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E24&amp;","&amp;F24&amp;","&amp;G24&amp;","&amp;H24&amp;","&amp;VLOOKUP(I24,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B24&amp;"'"&amp;","&amp;"'"&amp;C24&amp;"'"&amp;","&amp;VLOOKUP(D24,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E24&amp;","&amp;F24&amp;","&amp;G24&amp;","&amp;H24&amp;","&amp;VLOOKUP(I24,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster019','マジシャン',8,100,9,12,0.1,4);</v>
       </c>
     </row>
@@ -30465,7 +30495,7 @@
         <v>35</v>
       </c>
       <c r="L25" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B25&amp;"'"&amp;","&amp;"'"&amp;C25&amp;"'"&amp;","&amp;VLOOKUP(D25,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E25&amp;","&amp;F25&amp;","&amp;G25&amp;","&amp;H25&amp;","&amp;VLOOKUP(I25,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B25&amp;"'"&amp;","&amp;"'"&amp;C25&amp;"'"&amp;","&amp;VLOOKUP(D25,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E25&amp;","&amp;F25&amp;","&amp;G25&amp;","&amp;H25&amp;","&amp;VLOOKUP(I25,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster020','ウィザード',8,120,11,15,0.11,4);</v>
       </c>
     </row>
@@ -30498,7 +30528,7 @@
         <v>35</v>
       </c>
       <c r="L26" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B26&amp;"'"&amp;","&amp;"'"&amp;C26&amp;"'"&amp;","&amp;VLOOKUP(D26,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E26&amp;","&amp;F26&amp;","&amp;G26&amp;","&amp;H26&amp;","&amp;VLOOKUP(I26,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B26&amp;"'"&amp;","&amp;"'"&amp;C26&amp;"'"&amp;","&amp;VLOOKUP(D26,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E26&amp;","&amp;F26&amp;","&amp;G26&amp;","&amp;H26&amp;","&amp;VLOOKUP(I26,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster021','ハイウィザード',8,144,14,19,0.12,4);</v>
       </c>
     </row>
@@ -30528,7 +30558,7 @@
         <v>150</v>
       </c>
       <c r="L27" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B27&amp;"'"&amp;","&amp;"'"&amp;C27&amp;"'"&amp;","&amp;VLOOKUP(D27,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E27&amp;","&amp;F27&amp;","&amp;G27&amp;","&amp;H27&amp;","&amp;VLOOKUP(I27,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B27&amp;"'"&amp;","&amp;"'"&amp;C27&amp;"'"&amp;","&amp;VLOOKUP(D27,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E27&amp;","&amp;F27&amp;","&amp;G27&amp;","&amp;H27&amp;","&amp;VLOOKUP(I27,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster022','マイコニド',9,120,10,12,0.15,1);</v>
       </c>
     </row>
@@ -30561,7 +30591,7 @@
         <v>150</v>
       </c>
       <c r="L28" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B28&amp;"'"&amp;","&amp;"'"&amp;C28&amp;"'"&amp;","&amp;VLOOKUP(D28,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E28&amp;","&amp;F28&amp;","&amp;G28&amp;","&amp;H28&amp;","&amp;VLOOKUP(I28,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B28&amp;"'"&amp;","&amp;"'"&amp;C28&amp;"'"&amp;","&amp;VLOOKUP(D28,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E28&amp;","&amp;F28&amp;","&amp;G28&amp;","&amp;H28&amp;","&amp;VLOOKUP(I28,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster023','ダースマタンゴ',9,144,13,15,0.15,1);</v>
       </c>
     </row>
@@ -30591,7 +30621,7 @@
         <v>151</v>
       </c>
       <c r="L29" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B29&amp;"'"&amp;","&amp;"'"&amp;C29&amp;"'"&amp;","&amp;VLOOKUP(D29,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E29&amp;","&amp;F29&amp;","&amp;G29&amp;","&amp;H29&amp;","&amp;VLOOKUP(I29,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B29&amp;"'"&amp;","&amp;"'"&amp;C29&amp;"'"&amp;","&amp;VLOOKUP(D29,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E29&amp;","&amp;F29&amp;","&amp;G29&amp;","&amp;H29&amp;","&amp;VLOOKUP(I29,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster024','ニードルバード',10,100,13,16,0.25,3);</v>
       </c>
     </row>
@@ -30624,7 +30654,7 @@
         <v>151</v>
       </c>
       <c r="L30" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B30&amp;"'"&amp;","&amp;"'"&amp;C30&amp;"'"&amp;","&amp;VLOOKUP(D30,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E30&amp;","&amp;F30&amp;","&amp;G30&amp;","&amp;H30&amp;","&amp;VLOOKUP(I30,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B30&amp;"'"&amp;","&amp;"'"&amp;C30&amp;"'"&amp;","&amp;VLOOKUP(D30,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E30&amp;","&amp;F30&amp;","&amp;G30&amp;","&amp;H30&amp;","&amp;VLOOKUP(I30,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster025','コカトバード',10,120,16,20,0.27,3);</v>
       </c>
     </row>
@@ -30654,7 +30684,7 @@
         <v>151</v>
       </c>
       <c r="L31" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B31&amp;"'"&amp;","&amp;"'"&amp;C31&amp;"'"&amp;","&amp;VLOOKUP(D31,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E31&amp;","&amp;F31&amp;","&amp;G31&amp;","&amp;H31&amp;","&amp;VLOOKUP(I31,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B31&amp;"'"&amp;","&amp;"'"&amp;C31&amp;"'"&amp;","&amp;VLOOKUP(D31,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E31&amp;","&amp;F31&amp;","&amp;G31&amp;","&amp;H31&amp;","&amp;VLOOKUP(I31,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster026','プチドラゴン',11,130,13,8,0.08,3);</v>
       </c>
     </row>
@@ -30687,7 +30717,7 @@
         <v>36</v>
       </c>
       <c r="L32" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B32&amp;"'"&amp;","&amp;"'"&amp;C32&amp;"'"&amp;","&amp;VLOOKUP(D32,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E32&amp;","&amp;F32&amp;","&amp;G32&amp;","&amp;H32&amp;","&amp;VLOOKUP(I32,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B32&amp;"'"&amp;","&amp;"'"&amp;C32&amp;"'"&amp;","&amp;VLOOKUP(D32,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E32&amp;","&amp;F32&amp;","&amp;G32&amp;","&amp;H32&amp;","&amp;VLOOKUP(I32,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster027','プチドラゾンビ',11,156,16,10,0.1,5);</v>
       </c>
     </row>
@@ -30720,7 +30750,7 @@
         <v>150</v>
       </c>
       <c r="L33" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B33&amp;"'"&amp;","&amp;"'"&amp;C33&amp;"'"&amp;","&amp;VLOOKUP(D33,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E33&amp;","&amp;F33&amp;","&amp;G33&amp;","&amp;H33&amp;","&amp;VLOOKUP(I33,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B33&amp;"'"&amp;","&amp;"'"&amp;C33&amp;"'"&amp;","&amp;VLOOKUP(D33,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E33&amp;","&amp;F33&amp;","&amp;G33&amp;","&amp;H33&amp;","&amp;VLOOKUP(I33,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster028','フロストドラゴン',11,187,20,13,0.12,1);</v>
       </c>
     </row>
@@ -30753,7 +30783,7 @@
         <v>37</v>
       </c>
       <c r="L34" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B34&amp;"'"&amp;","&amp;"'"&amp;C34&amp;"'"&amp;","&amp;VLOOKUP(D34,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E34&amp;","&amp;F34&amp;","&amp;G34&amp;","&amp;H34&amp;","&amp;VLOOKUP(I34,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B34&amp;"'"&amp;","&amp;"'"&amp;C34&amp;"'"&amp;","&amp;VLOOKUP(D34,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E34&amp;","&amp;F34&amp;","&amp;G34&amp;","&amp;H34&amp;","&amp;VLOOKUP(I34,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster029','プチティアマット',11,224,26,16,0.13,6);</v>
       </c>
     </row>
@@ -30783,7 +30813,7 @@
         <v>37</v>
       </c>
       <c r="L35" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B35&amp;"'"&amp;","&amp;"'"&amp;C35&amp;"'"&amp;","&amp;VLOOKUP(D35,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E35&amp;","&amp;F35&amp;","&amp;G35&amp;","&amp;H35&amp;","&amp;VLOOKUP(I35,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B35&amp;"'"&amp;","&amp;"'"&amp;C35&amp;"'"&amp;","&amp;VLOOKUP(D35,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E35&amp;","&amp;F35&amp;","&amp;G35&amp;","&amp;H35&amp;","&amp;VLOOKUP(I35,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster030','ポト',12,100,10,16,0.18,6);</v>
       </c>
     </row>
@@ -30816,7 +30846,7 @@
         <v>37</v>
       </c>
       <c r="L36" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B36&amp;"'"&amp;","&amp;"'"&amp;C36&amp;"'"&amp;","&amp;VLOOKUP(D36,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E36&amp;","&amp;F36&amp;","&amp;G36&amp;","&amp;H36&amp;","&amp;VLOOKUP(I36,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B36&amp;"'"&amp;","&amp;"'"&amp;C36&amp;"'"&amp;","&amp;VLOOKUP(D36,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E36&amp;","&amp;F36&amp;","&amp;G36&amp;","&amp;H36&amp;","&amp;VLOOKUP(I36,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster031','マーマポト',12,120,13,20,0.2,6);</v>
       </c>
     </row>
@@ -30849,7 +30879,7 @@
         <v>37</v>
       </c>
       <c r="L37" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B37&amp;"'"&amp;","&amp;"'"&amp;C37&amp;"'"&amp;","&amp;VLOOKUP(D37,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E37&amp;","&amp;F37&amp;","&amp;G37&amp;","&amp;H37&amp;","&amp;VLOOKUP(I37,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B37&amp;"'"&amp;","&amp;"'"&amp;C37&amp;"'"&amp;","&amp;VLOOKUP(D37,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E37&amp;","&amp;F37&amp;","&amp;G37&amp;","&amp;H37&amp;","&amp;VLOOKUP(I37,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster032','パーパポト',12,141,16,26,0.22,6);</v>
       </c>
     </row>
@@ -30879,7 +30909,7 @@
         <v>37</v>
       </c>
       <c r="L38" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B38&amp;"'"&amp;","&amp;"'"&amp;C38&amp;"'"&amp;","&amp;VLOOKUP(D38,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E38&amp;","&amp;F38&amp;","&amp;G38&amp;","&amp;H38&amp;","&amp;VLOOKUP(I38,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B38&amp;"'"&amp;","&amp;"'"&amp;C38&amp;"'"&amp;","&amp;VLOOKUP(D38,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E38&amp;","&amp;F38&amp;","&amp;G38&amp;","&amp;H38&amp;","&amp;VLOOKUP(I38,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster033','プリースト',13,100,9,13,0.1,6);</v>
       </c>
     </row>
@@ -30912,7 +30942,7 @@
         <v>36</v>
       </c>
       <c r="L39" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B39&amp;"'"&amp;","&amp;"'"&amp;C39&amp;"'"&amp;","&amp;VLOOKUP(D39,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E39&amp;","&amp;F39&amp;","&amp;G39&amp;","&amp;H39&amp;","&amp;VLOOKUP(I39,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B39&amp;"'"&amp;","&amp;"'"&amp;C39&amp;"'"&amp;","&amp;VLOOKUP(D39,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E39&amp;","&amp;F39&amp;","&amp;G39&amp;","&amp;H39&amp;","&amp;VLOOKUP(I39,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster034','カオスソーサラー',13,120,11,16,0.11,5);</v>
       </c>
     </row>
@@ -30945,7 +30975,7 @@
         <v>36</v>
       </c>
       <c r="L40" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B40&amp;"'"&amp;","&amp;"'"&amp;C40&amp;"'"&amp;","&amp;VLOOKUP(D40,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E40&amp;","&amp;F40&amp;","&amp;G40&amp;","&amp;H40&amp;","&amp;VLOOKUP(I40,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B40&amp;"'"&amp;","&amp;"'"&amp;C40&amp;"'"&amp;","&amp;VLOOKUP(D40,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E40&amp;","&amp;F40&amp;","&amp;G40&amp;","&amp;H40&amp;","&amp;VLOOKUP(I40,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster035','イビルシャーマン',13,144,14,20,0.13,5);</v>
       </c>
     </row>
@@ -30976,7 +31006,7 @@
         <v>37</v>
       </c>
       <c r="L41" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B41&amp;"'"&amp;","&amp;"'"&amp;C41&amp;"'"&amp;","&amp;VLOOKUP(D41,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E41&amp;","&amp;F41&amp;","&amp;G41&amp;","&amp;H41&amp;","&amp;VLOOKUP(I41,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B41&amp;"'"&amp;","&amp;"'"&amp;C41&amp;"'"&amp;","&amp;VLOOKUP(D41,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E41&amp;","&amp;F41&amp;","&amp;G41&amp;","&amp;H41&amp;","&amp;VLOOKUP(I41,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster036','ラビ',14,100,11,16,0.16,6);</v>
       </c>
     </row>
@@ -31009,7 +31039,7 @@
         <v>37</v>
       </c>
       <c r="L42" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B42&amp;"'"&amp;","&amp;"'"&amp;C42&amp;"'"&amp;","&amp;VLOOKUP(D42,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E42&amp;","&amp;F42&amp;","&amp;G42&amp;","&amp;H42&amp;","&amp;VLOOKUP(I42,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B42&amp;"'"&amp;","&amp;"'"&amp;C42&amp;"'"&amp;","&amp;VLOOKUP(D42,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E42&amp;","&amp;F42&amp;","&amp;G42&amp;","&amp;H42&amp;","&amp;VLOOKUP(I42,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster037','ラビリオン',14,120,14,20,0.17,6);</v>
       </c>
     </row>
@@ -31042,7 +31072,7 @@
         <v>37</v>
       </c>
       <c r="L43" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B43&amp;"'"&amp;","&amp;"'"&amp;C43&amp;"'"&amp;","&amp;VLOOKUP(D43,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E43&amp;","&amp;F43&amp;","&amp;G43&amp;","&amp;H43&amp;","&amp;VLOOKUP(I43,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B43&amp;"'"&amp;","&amp;"'"&amp;C43&amp;"'"&amp;","&amp;VLOOKUP(D43,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E43&amp;","&amp;F43&amp;","&amp;G43&amp;","&amp;H43&amp;","&amp;VLOOKUP(I43,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster038','キングラビ',14,144,18,26,0.18,6);</v>
       </c>
     </row>
@@ -31075,7 +31105,7 @@
         <v>37</v>
       </c>
       <c r="L44" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B44&amp;"'"&amp;","&amp;"'"&amp;C44&amp;"'"&amp;","&amp;VLOOKUP(D44,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E44&amp;","&amp;F44&amp;","&amp;G44&amp;","&amp;H44&amp;","&amp;VLOOKUP(I44,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B44&amp;"'"&amp;","&amp;"'"&amp;C44&amp;"'"&amp;","&amp;VLOOKUP(D44,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E44&amp;","&amp;F44&amp;","&amp;G44&amp;","&amp;H44&amp;","&amp;VLOOKUP(I44,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster039','グレートラビ',14,172,23,33,0.2,6);</v>
       </c>
     </row>
@@ -31105,7 +31135,7 @@
         <v>34</v>
       </c>
       <c r="L45" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B45&amp;"'"&amp;","&amp;"'"&amp;C45&amp;"'"&amp;","&amp;VLOOKUP(D45,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E45&amp;","&amp;F45&amp;","&amp;G45&amp;","&amp;H45&amp;","&amp;VLOOKUP(I45,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B45&amp;"'"&amp;","&amp;"'"&amp;C45&amp;"'"&amp;","&amp;VLOOKUP(D45,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E45&amp;","&amp;F45&amp;","&amp;G45&amp;","&amp;H45&amp;","&amp;VLOOKUP(I45,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster040','スライム',15,100,10,18,0.15,2);</v>
       </c>
     </row>
@@ -31138,7 +31168,7 @@
         <v>150</v>
       </c>
       <c r="L46" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B46&amp;"'"&amp;","&amp;"'"&amp;C46&amp;"'"&amp;","&amp;VLOOKUP(D46,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E46&amp;","&amp;F46&amp;","&amp;G46&amp;","&amp;H46&amp;","&amp;VLOOKUP(I46,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B46&amp;"'"&amp;","&amp;"'"&amp;C46&amp;"'"&amp;","&amp;VLOOKUP(D46,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E46&amp;","&amp;F46&amp;","&amp;G46&amp;","&amp;H46&amp;","&amp;VLOOKUP(I46,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster041','ブルーババロア',15,120,13,23,0.15,1);</v>
       </c>
     </row>
@@ -31171,7 +31201,7 @@
         <v>151</v>
       </c>
       <c r="L47" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B47&amp;"'"&amp;","&amp;"'"&amp;C47&amp;"'"&amp;","&amp;VLOOKUP(D47,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E47&amp;","&amp;F47&amp;","&amp;G47&amp;","&amp;H47&amp;","&amp;VLOOKUP(I47,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B47&amp;"'"&amp;","&amp;"'"&amp;C47&amp;"'"&amp;","&amp;VLOOKUP(D47,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E47&amp;","&amp;F47&amp;","&amp;G47&amp;","&amp;H47&amp;","&amp;VLOOKUP(I47,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster042','レッドマシュマロ',15,141,16,29,0.15,3);</v>
       </c>
     </row>
@@ -31201,7 +31231,7 @@
         <v>36</v>
       </c>
       <c r="L48" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B48&amp;"'"&amp;","&amp;"'"&amp;C48&amp;"'"&amp;","&amp;VLOOKUP(D48,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E48&amp;","&amp;F48&amp;","&amp;G48&amp;","&amp;H48&amp;","&amp;VLOOKUP(I48,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B48&amp;"'"&amp;","&amp;"'"&amp;C48&amp;"'"&amp;","&amp;VLOOKUP(D48,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E48&amp;","&amp;F48&amp;","&amp;G48&amp;","&amp;H48&amp;","&amp;VLOOKUP(I48,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster043','イビルソード',16,110,15,13,0.14,5);</v>
       </c>
     </row>
@@ -31234,7 +31264,7 @@
         <v>36</v>
       </c>
       <c r="L49" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B49&amp;"'"&amp;","&amp;"'"&amp;C49&amp;"'"&amp;","&amp;VLOOKUP(D49,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E49&amp;","&amp;F49&amp;","&amp;G49&amp;","&amp;H49&amp;","&amp;VLOOKUP(I49,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B49&amp;"'"&amp;","&amp;"'"&amp;C49&amp;"'"&amp;","&amp;VLOOKUP(D49,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E49&amp;","&amp;F49&amp;","&amp;G49&amp;","&amp;H49&amp;","&amp;VLOOKUP(I49,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster044','イビルウェポン',16,132,19,16,0.15,5);</v>
       </c>
     </row>
@@ -31267,7 +31297,7 @@
         <v>37</v>
       </c>
       <c r="L50" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B50&amp;"'"&amp;","&amp;"'"&amp;C50&amp;"'"&amp;","&amp;VLOOKUP(D50,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E50&amp;","&amp;F50&amp;","&amp;G50&amp;","&amp;H50&amp;","&amp;VLOOKUP(I50,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B50&amp;"'"&amp;","&amp;"'"&amp;C50&amp;"'"&amp;","&amp;VLOOKUP(D50,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E50&amp;","&amp;F50&amp;","&amp;G50&amp;","&amp;H50&amp;","&amp;VLOOKUP(I50,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster045','エレメントソード',16,158,24,20,0.16,6);</v>
       </c>
     </row>
@@ -31297,7 +31327,7 @@
         <v>150</v>
       </c>
       <c r="L51" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B51&amp;"'"&amp;","&amp;"'"&amp;C51&amp;"'"&amp;","&amp;VLOOKUP(D51,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E51&amp;","&amp;F51&amp;","&amp;G51&amp;","&amp;H51&amp;","&amp;VLOOKUP(I51,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B51&amp;"'"&amp;","&amp;"'"&amp;C51&amp;"'"&amp;","&amp;VLOOKUP(D51,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E51&amp;","&amp;F51&amp;","&amp;G51&amp;","&amp;H51&amp;","&amp;VLOOKUP(I51,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster046','ケルベロス',17,110,11,19,0.18,1);</v>
       </c>
     </row>
@@ -31330,7 +31360,7 @@
         <v>150</v>
       </c>
       <c r="L52" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B52&amp;"'"&amp;","&amp;"'"&amp;C52&amp;"'"&amp;","&amp;VLOOKUP(D52,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E52&amp;","&amp;F52&amp;","&amp;G52&amp;","&amp;H52&amp;","&amp;VLOOKUP(I52,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B52&amp;"'"&amp;","&amp;"'"&amp;C52&amp;"'"&amp;","&amp;VLOOKUP(D52,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E52&amp;","&amp;F52&amp;","&amp;G52&amp;","&amp;H52&amp;","&amp;VLOOKUP(I52,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster047','バウンドウルフ',17,132,14,24,0.2,1);</v>
       </c>
     </row>
@@ -31363,7 +31393,7 @@
         <v>150</v>
       </c>
       <c r="L53" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B53&amp;"'"&amp;","&amp;"'"&amp;C53&amp;"'"&amp;","&amp;VLOOKUP(D53,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E53&amp;","&amp;F53&amp;","&amp;G53&amp;","&amp;H53&amp;","&amp;VLOOKUP(I53,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B53&amp;"'"&amp;","&amp;"'"&amp;C53&amp;"'"&amp;","&amp;VLOOKUP(D53,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E53&amp;","&amp;F53&amp;","&amp;G53&amp;","&amp;H53&amp;","&amp;VLOOKUP(I53,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster048','ジャッカル',17,158,18,31,0.21,1);</v>
       </c>
     </row>
@@ -31393,7 +31423,7 @@
         <v>151</v>
       </c>
       <c r="L54" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B54&amp;"'"&amp;","&amp;"'"&amp;C54&amp;"'"&amp;","&amp;VLOOKUP(D54,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E54&amp;","&amp;F54&amp;","&amp;G54&amp;","&amp;H54&amp;","&amp;VLOOKUP(I54,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B54&amp;"'"&amp;","&amp;"'"&amp;C54&amp;"'"&amp;","&amp;VLOOKUP(D54,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E54&amp;","&amp;F54&amp;","&amp;G54&amp;","&amp;H54&amp;","&amp;VLOOKUP(I54,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster049','ダックソルジャー',18,120,16,14,0.15,3);</v>
       </c>
     </row>
@@ -31423,7 +31453,7 @@
         <v>151</v>
       </c>
       <c r="L55" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B55&amp;"'"&amp;","&amp;"'"&amp;C55&amp;"'"&amp;","&amp;VLOOKUP(D55,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E55&amp;","&amp;F55&amp;","&amp;G55&amp;","&amp;H55&amp;","&amp;VLOOKUP(I55,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B55&amp;"'"&amp;","&amp;"'"&amp;C55&amp;"'"&amp;","&amp;VLOOKUP(D55,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E55&amp;","&amp;F55&amp;","&amp;G55&amp;","&amp;H55&amp;","&amp;VLOOKUP(I55,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster050','ダックジェネラル',18,160,24,20,0.15,3);</v>
       </c>
     </row>
@@ -31453,7 +31483,7 @@
         <v>34</v>
       </c>
       <c r="L56" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B56&amp;"'"&amp;","&amp;"'"&amp;C56&amp;"'"&amp;","&amp;VLOOKUP(D56,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E56&amp;","&amp;F56&amp;","&amp;G56&amp;","&amp;H56&amp;","&amp;VLOOKUP(I56,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B56&amp;"'"&amp;","&amp;"'"&amp;C56&amp;"'"&amp;","&amp;VLOOKUP(D56,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E56&amp;","&amp;F56&amp;","&amp;G56&amp;","&amp;H56&amp;","&amp;VLOOKUP(I56,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster051','モールベア',19,130,14,18,0.18,2);</v>
       </c>
     </row>
@@ -31483,7 +31513,7 @@
         <v>34</v>
       </c>
       <c r="L57" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B57&amp;"'"&amp;","&amp;"'"&amp;C57&amp;"'"&amp;","&amp;VLOOKUP(D57,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E57&amp;","&amp;F57&amp;","&amp;G57&amp;","&amp;H57&amp;","&amp;VLOOKUP(I57,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B57&amp;"'"&amp;","&amp;"'"&amp;C57&amp;"'"&amp;","&amp;VLOOKUP(D57,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E57&amp;","&amp;F57&amp;","&amp;G57&amp;","&amp;H57&amp;","&amp;VLOOKUP(I57,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster052','ニードリオン',19,170,18,26,0.2,2);</v>
       </c>
     </row>
@@ -31513,7 +31543,7 @@
         <v>35</v>
       </c>
       <c r="L58" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B58&amp;"'"&amp;","&amp;"'"&amp;C58&amp;"'"&amp;","&amp;VLOOKUP(D58,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E58&amp;","&amp;F58&amp;","&amp;G58&amp;","&amp;H58&amp;","&amp;VLOOKUP(I58,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B58&amp;"'"&amp;","&amp;"'"&amp;C58&amp;"'"&amp;","&amp;VLOOKUP(D58,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E58&amp;","&amp;F58&amp;","&amp;G58&amp;","&amp;H58&amp;","&amp;VLOOKUP(I58,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster053','ギャルビー',20,120,13,16,0.2,4);</v>
       </c>
     </row>
@@ -31546,7 +31576,7 @@
         <v>35</v>
       </c>
       <c r="L59" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B59&amp;"'"&amp;","&amp;"'"&amp;C59&amp;"'"&amp;","&amp;VLOOKUP(D59,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E59&amp;","&amp;F59&amp;","&amp;G59&amp;","&amp;H59&amp;","&amp;VLOOKUP(I59,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B59&amp;"'"&amp;","&amp;"'"&amp;C59&amp;"'"&amp;","&amp;VLOOKUP(D59,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E59&amp;","&amp;F59&amp;","&amp;G59&amp;","&amp;H59&amp;","&amp;VLOOKUP(I59,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster054','レディビー',20,144,16,20,0.22,4);</v>
       </c>
     </row>
@@ -31579,7 +31609,7 @@
         <v>35</v>
       </c>
       <c r="L60" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B60&amp;"'"&amp;","&amp;"'"&amp;C60&amp;"'"&amp;","&amp;VLOOKUP(D60,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E60&amp;","&amp;F60&amp;","&amp;G60&amp;","&amp;H60&amp;","&amp;VLOOKUP(I60,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B60&amp;"'"&amp;","&amp;"'"&amp;C60&amp;"'"&amp;","&amp;VLOOKUP(D60,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E60&amp;","&amp;F60&amp;","&amp;G60&amp;","&amp;H60&amp;","&amp;VLOOKUP(I60,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster055','クインビー',20,172,20,26,0.23,4);</v>
       </c>
     </row>
@@ -31609,7 +31639,7 @@
         <v>150</v>
       </c>
       <c r="L61" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B61&amp;"'"&amp;","&amp;"'"&amp;C61&amp;"'"&amp;","&amp;VLOOKUP(D61,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E61&amp;","&amp;F61&amp;","&amp;G61&amp;","&amp;H61&amp;","&amp;VLOOKUP(I61,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B61&amp;"'"&amp;","&amp;"'"&amp;C61&amp;"'"&amp;","&amp;VLOOKUP(D61,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E61&amp;","&amp;F61&amp;","&amp;G61&amp;","&amp;H61&amp;","&amp;VLOOKUP(I61,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster056','サハギン',21,130,16,16,0.15,1);</v>
       </c>
     </row>
@@ -31639,7 +31669,7 @@
         <v>150</v>
       </c>
       <c r="L62" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B62&amp;"'"&amp;","&amp;"'"&amp;C62&amp;"'"&amp;","&amp;VLOOKUP(D62,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E62&amp;","&amp;F62&amp;","&amp;G62&amp;","&amp;H62&amp;","&amp;VLOOKUP(I62,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B62&amp;"'"&amp;","&amp;"'"&amp;C62&amp;"'"&amp;","&amp;VLOOKUP(D62,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E62&amp;","&amp;F62&amp;","&amp;G62&amp;","&amp;H62&amp;","&amp;VLOOKUP(I62,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster057','プチポセイドン',21,150,22,19,0.15,1);</v>
       </c>
     </row>
@@ -31669,7 +31699,7 @@
         <v>298</v>
       </c>
       <c r="L63" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B63&amp;"'"&amp;","&amp;"'"&amp;C63&amp;"'"&amp;","&amp;VLOOKUP(D63,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E63&amp;","&amp;F63&amp;","&amp;G63&amp;","&amp;H63&amp;","&amp;VLOOKUP(I63,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B63&amp;"'"&amp;","&amp;"'"&amp;C63&amp;"'"&amp;","&amp;VLOOKUP(D63,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E63&amp;","&amp;F63&amp;","&amp;G63&amp;","&amp;H63&amp;","&amp;VLOOKUP(I63,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster058','クロウラー',22,130,15,11,0.08,2);</v>
       </c>
     </row>
@@ -31702,7 +31732,7 @@
         <v>34</v>
       </c>
       <c r="L64" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B64&amp;"'"&amp;","&amp;"'"&amp;C64&amp;"'"&amp;","&amp;VLOOKUP(D64,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E64&amp;","&amp;F64&amp;","&amp;G64&amp;","&amp;H64&amp;","&amp;VLOOKUP(I64,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B64&amp;"'"&amp;","&amp;"'"&amp;C64&amp;"'"&amp;","&amp;VLOOKUP(D64,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E64&amp;","&amp;F64&amp;","&amp;G64&amp;","&amp;H64&amp;","&amp;VLOOKUP(I64,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster059','メガクロウラー',22,156,19,14,0.09,2);</v>
       </c>
     </row>
@@ -31735,7 +31765,7 @@
         <v>34</v>
       </c>
       <c r="L65" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B65&amp;"'"&amp;","&amp;"'"&amp;C65&amp;"'"&amp;","&amp;VLOOKUP(D65,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E65&amp;","&amp;F65&amp;","&amp;G65&amp;","&amp;H65&amp;","&amp;VLOOKUP(I65,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B65&amp;"'"&amp;","&amp;"'"&amp;C65&amp;"'"&amp;","&amp;VLOOKUP(D65,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E65&amp;","&amp;F65&amp;","&amp;G65&amp;","&amp;H65&amp;","&amp;VLOOKUP(I65,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster060','ギガクロウラー',22,187,24,18,0.1,2);</v>
       </c>
     </row>
@@ -31765,7 +31795,7 @@
         <v>34</v>
       </c>
       <c r="L66" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B66&amp;"'"&amp;","&amp;"'"&amp;C66&amp;"'"&amp;","&amp;VLOOKUP(D66,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E66&amp;","&amp;F66&amp;","&amp;G66&amp;","&amp;H66&amp;","&amp;VLOOKUP(I66,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B66&amp;"'"&amp;","&amp;"'"&amp;C66&amp;"'"&amp;","&amp;VLOOKUP(D66,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E66&amp;","&amp;F66&amp;","&amp;G66&amp;","&amp;H66&amp;","&amp;VLOOKUP(I66,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster061','ぱっくんオタマ',23,110,12,10,0.15,2);</v>
       </c>
     </row>
@@ -31798,7 +31828,7 @@
         <v>34</v>
       </c>
       <c r="L67" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B67&amp;"'"&amp;","&amp;"'"&amp;C67&amp;"'"&amp;","&amp;VLOOKUP(D67,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E67&amp;","&amp;F67&amp;","&amp;G67&amp;","&amp;H67&amp;","&amp;VLOOKUP(I67,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B67&amp;"'"&amp;","&amp;"'"&amp;C67&amp;"'"&amp;","&amp;VLOOKUP(D67,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E67&amp;","&amp;F67&amp;","&amp;G67&amp;","&amp;H67&amp;","&amp;VLOOKUP(I67,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster062','ぱっくりオタマ',23,132,15,13,0.15,2);</v>
       </c>
     </row>
@@ -31831,7 +31861,7 @@
         <v>151</v>
       </c>
       <c r="L68" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B68&amp;"'"&amp;","&amp;"'"&amp;C68&amp;"'"&amp;","&amp;VLOOKUP(D68,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E68&amp;","&amp;F68&amp;","&amp;G68&amp;","&amp;H68&amp;","&amp;VLOOKUP(I68,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B68&amp;"'"&amp;","&amp;"'"&amp;C68&amp;"'"&amp;","&amp;VLOOKUP(D68,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E68&amp;","&amp;F68&amp;","&amp;G68&amp;","&amp;H68&amp;","&amp;VLOOKUP(I68,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster063','ぱっくんトカゲ',23,158,19,16,0.1,3);</v>
       </c>
     </row>
@@ -31864,7 +31894,7 @@
         <v>151</v>
       </c>
       <c r="L69" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B69&amp;"'"&amp;","&amp;"'"&amp;C69&amp;"'"&amp;","&amp;VLOOKUP(D69,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E69&amp;","&amp;F69&amp;","&amp;G69&amp;","&amp;H69&amp;","&amp;VLOOKUP(I69,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B69&amp;"'"&amp;","&amp;"'"&amp;C69&amp;"'"&amp;","&amp;VLOOKUP(D69,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E69&amp;","&amp;F69&amp;","&amp;G69&amp;","&amp;H69&amp;","&amp;VLOOKUP(I69,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster064','ぱっくんドラゴン',23,189,24,20,0.11,3);</v>
       </c>
     </row>
@@ -31894,7 +31924,7 @@
         <v>36</v>
       </c>
       <c r="L70" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B70&amp;"'"&amp;","&amp;"'"&amp;C70&amp;"'"&amp;","&amp;VLOOKUP(D70,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E70&amp;","&amp;F70&amp;","&amp;G70&amp;","&amp;H70&amp;","&amp;VLOOKUP(I70,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B70&amp;"'"&amp;","&amp;"'"&amp;C70&amp;"'"&amp;","&amp;VLOOKUP(D70,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E70&amp;","&amp;F70&amp;","&amp;G70&amp;","&amp;H70&amp;","&amp;VLOOKUP(I70,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster065','チビデビル',24,120,13,17,0.22,5);</v>
       </c>
     </row>
@@ -31924,7 +31954,7 @@
         <v>36</v>
       </c>
       <c r="L71" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B71&amp;"'"&amp;","&amp;"'"&amp;C71&amp;"'"&amp;","&amp;VLOOKUP(D71,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E71&amp;","&amp;F71&amp;","&amp;G71&amp;","&amp;H71&amp;","&amp;VLOOKUP(I71,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B71&amp;"'"&amp;","&amp;"'"&amp;C71&amp;"'"&amp;","&amp;VLOOKUP(D71,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E71&amp;","&amp;F71&amp;","&amp;G71&amp;","&amp;H71&amp;","&amp;VLOOKUP(I71,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster066','グレムリン',24,160,18,20,0.24,5);</v>
       </c>
     </row>
@@ -31954,7 +31984,7 @@
         <v>36</v>
       </c>
       <c r="L72" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B72&amp;"'"&amp;","&amp;"'"&amp;C72&amp;"'"&amp;","&amp;VLOOKUP(D72,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E72&amp;","&amp;F72&amp;","&amp;G72&amp;","&amp;H72&amp;","&amp;VLOOKUP(I72,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B72&amp;"'"&amp;","&amp;"'"&amp;C72&amp;"'"&amp;","&amp;VLOOKUP(D72,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E72&amp;","&amp;F72&amp;","&amp;G72&amp;","&amp;H72&amp;","&amp;VLOOKUP(I72,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster067','オーガボックス',25,140,18,17,0.15,5);</v>
       </c>
     </row>
@@ -31984,7 +32014,7 @@
         <v>36</v>
       </c>
       <c r="L73" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B73&amp;"'"&amp;","&amp;"'"&amp;C73&amp;"'"&amp;","&amp;VLOOKUP(D73,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E73&amp;","&amp;F73&amp;","&amp;G73&amp;","&amp;H73&amp;","&amp;VLOOKUP(I73,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B73&amp;"'"&amp;","&amp;"'"&amp;C73&amp;"'"&amp;","&amp;VLOOKUP(D73,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E73&amp;","&amp;F73&amp;","&amp;G73&amp;","&amp;H73&amp;","&amp;VLOOKUP(I73,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster068','カイザーミミック',25,170,23,20,0.15,5);</v>
       </c>
     </row>
@@ -32014,7 +32044,7 @@
         <v>151</v>
       </c>
       <c r="L74" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B74&amp;"'"&amp;","&amp;"'"&amp;C74&amp;"'"&amp;","&amp;VLOOKUP(D74,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E74&amp;","&amp;F74&amp;","&amp;G74&amp;","&amp;H74&amp;","&amp;VLOOKUP(I74,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B74&amp;"'"&amp;","&amp;"'"&amp;C74&amp;"'"&amp;","&amp;VLOOKUP(D74,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E74&amp;","&amp;F74&amp;","&amp;G74&amp;","&amp;H74&amp;","&amp;VLOOKUP(I74,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster069','バレッテ',26,140,15,12,0.05,3);</v>
       </c>
     </row>
@@ -32044,7 +32074,7 @@
         <v>151</v>
       </c>
       <c r="L75" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B75&amp;"'"&amp;","&amp;"'"&amp;C75&amp;"'"&amp;","&amp;VLOOKUP(D75,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E75&amp;","&amp;F75&amp;","&amp;G75&amp;","&amp;H75&amp;","&amp;VLOOKUP(I75,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B75&amp;"'"&amp;","&amp;"'"&amp;C75&amp;"'"&amp;","&amp;VLOOKUP(D75,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E75&amp;","&amp;F75&amp;","&amp;G75&amp;","&amp;H75&amp;","&amp;VLOOKUP(I75,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster070','ゴールドバレッテ',26,180,19,14,0.05,3);</v>
       </c>
     </row>
@@ -32074,7 +32104,7 @@
         <v>34</v>
       </c>
       <c r="L76" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B76&amp;"'"&amp;","&amp;"'"&amp;C76&amp;"'"&amp;","&amp;VLOOKUP(D76,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E76&amp;","&amp;F76&amp;","&amp;G76&amp;","&amp;H76&amp;","&amp;VLOOKUP(I76,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B76&amp;"'"&amp;","&amp;"'"&amp;C76&amp;"'"&amp;","&amp;VLOOKUP(D76,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E76&amp;","&amp;F76&amp;","&amp;G76&amp;","&amp;H76&amp;","&amp;VLOOKUP(I76,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster071','バシリスク',27,110,12,15,0.15,2);</v>
       </c>
     </row>
@@ -32104,7 +32134,7 @@
         <v>151</v>
       </c>
       <c r="L77" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B77&amp;"'"&amp;","&amp;"'"&amp;C77&amp;"'"&amp;","&amp;VLOOKUP(D77,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E77&amp;","&amp;F77&amp;","&amp;G77&amp;","&amp;H77&amp;","&amp;VLOOKUP(I77,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B77&amp;"'"&amp;","&amp;"'"&amp;C77&amp;"'"&amp;","&amp;VLOOKUP(D77,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E77&amp;","&amp;F77&amp;","&amp;G77&amp;","&amp;H77&amp;","&amp;VLOOKUP(I77,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster072','ファイアドレイク',27,150,18,22,0.18,3);</v>
       </c>
     </row>
@@ -32134,7 +32164,7 @@
         <v>36</v>
       </c>
       <c r="L78" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B78&amp;"'"&amp;","&amp;"'"&amp;C78&amp;"'"&amp;","&amp;VLOOKUP(D78,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E78&amp;","&amp;F78&amp;","&amp;G78&amp;","&amp;H78&amp;","&amp;VLOOKUP(I78,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B78&amp;"'"&amp;","&amp;"'"&amp;C78&amp;"'"&amp;","&amp;VLOOKUP(D78,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E78&amp;","&amp;F78&amp;","&amp;G78&amp;","&amp;H78&amp;","&amp;VLOOKUP(I78,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster073','スペクター',28,130,13,17,0.2,5);</v>
       </c>
     </row>
@@ -32164,7 +32194,7 @@
         <v>36</v>
       </c>
       <c r="L79" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B79&amp;"'"&amp;","&amp;"'"&amp;C79&amp;"'"&amp;","&amp;VLOOKUP(D79,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E79&amp;","&amp;F79&amp;","&amp;G79&amp;","&amp;H79&amp;","&amp;VLOOKUP(I79,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B79&amp;"'"&amp;","&amp;"'"&amp;C79&amp;"'"&amp;","&amp;VLOOKUP(D79,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E79&amp;","&amp;F79&amp;","&amp;G79&amp;","&amp;H79&amp;","&amp;VLOOKUP(I79,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster074','ゴースト',28,160,17,20,0.21,5);</v>
       </c>
     </row>
@@ -32194,7 +32224,7 @@
         <v>37</v>
       </c>
       <c r="L80" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B80&amp;"'"&amp;","&amp;"'"&amp;C80&amp;"'"&amp;","&amp;VLOOKUP(D80,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E80&amp;","&amp;F80&amp;","&amp;G80&amp;","&amp;H80&amp;","&amp;VLOOKUP(I80,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B80&amp;"'"&amp;","&amp;"'"&amp;C80&amp;"'"&amp;","&amp;VLOOKUP(D80,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E80&amp;","&amp;F80&amp;","&amp;G80&amp;","&amp;H80&amp;","&amp;VLOOKUP(I80,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster075','ユニコーンヘッド',29,120,15,14,0.15,6);</v>
       </c>
     </row>
@@ -32224,7 +32254,7 @@
         <v>37</v>
       </c>
       <c r="L81" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B81&amp;"'"&amp;","&amp;"'"&amp;C81&amp;"'"&amp;","&amp;VLOOKUP(D81,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E81&amp;","&amp;F81&amp;","&amp;G81&amp;","&amp;H81&amp;","&amp;VLOOKUP(I81,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B81&amp;"'"&amp;","&amp;"'"&amp;C81&amp;"'"&amp;","&amp;VLOOKUP(D81,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E81&amp;","&amp;F81&amp;","&amp;G81&amp;","&amp;H81&amp;","&amp;VLOOKUP(I81,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster076','ゴールドユニコ',29,170,22,25,0.15,6);</v>
       </c>
     </row>
@@ -32254,7 +32284,7 @@
         <v>36</v>
       </c>
       <c r="L82" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B82&amp;"'"&amp;","&amp;"'"&amp;C82&amp;"'"&amp;","&amp;VLOOKUP(D82,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E82&amp;","&amp;F82&amp;","&amp;G82&amp;","&amp;H82&amp;","&amp;VLOOKUP(I82,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B82&amp;"'"&amp;","&amp;"'"&amp;C82&amp;"'"&amp;","&amp;VLOOKUP(D82,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E82&amp;","&amp;F82&amp;","&amp;G82&amp;","&amp;H82&amp;","&amp;VLOOKUP(I82,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster077','シェイプシフター',30,130,12,14,0.14,5);</v>
       </c>
     </row>
@@ -32286,7 +32316,7 @@
         <v>36</v>
       </c>
       <c r="L83" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B83&amp;"'"&amp;","&amp;"'"&amp;C83&amp;"'"&amp;","&amp;VLOOKUP(D83,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E83&amp;","&amp;F83&amp;","&amp;G83&amp;","&amp;H83&amp;","&amp;VLOOKUP(I83,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B83&amp;"'"&amp;","&amp;"'"&amp;C83&amp;"'"&amp;","&amp;VLOOKUP(D83,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E83&amp;","&amp;F83&amp;","&amp;G83&amp;","&amp;H83&amp;","&amp;VLOOKUP(I83,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster078','シャドウゼロ',30,170,15,18,0.15,5);</v>
       </c>
     </row>
@@ -32318,7 +32348,7 @@
         <v>36</v>
       </c>
       <c r="L84" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B84&amp;"'"&amp;","&amp;"'"&amp;C84&amp;"'"&amp;","&amp;VLOOKUP(D84,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E84&amp;","&amp;F84&amp;","&amp;G84&amp;","&amp;H84&amp;","&amp;VLOOKUP(I84,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B84&amp;"'"&amp;","&amp;"'"&amp;C84&amp;"'"&amp;","&amp;VLOOKUP(D84,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E84&amp;","&amp;F84&amp;","&amp;G84&amp;","&amp;H84&amp;","&amp;VLOOKUP(I84,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster079','シャドウゼロワン',30,190,19,23,0.16,5);</v>
       </c>
     </row>
@@ -32348,7 +32378,7 @@
         <v>36</v>
       </c>
       <c r="L85" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B85&amp;"'"&amp;","&amp;"'"&amp;C85&amp;"'"&amp;","&amp;VLOOKUP(D85,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E85&amp;","&amp;F85&amp;","&amp;G85&amp;","&amp;H85&amp;","&amp;VLOOKUP(I85,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B85&amp;"'"&amp;","&amp;"'"&amp;C85&amp;"'"&amp;","&amp;VLOOKUP(D85,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E85&amp;","&amp;F85&amp;","&amp;G85&amp;","&amp;H85&amp;","&amp;VLOOKUP(I85,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster080','ボルダー',31,120,13,14,0.25,5);</v>
       </c>
     </row>
@@ -32381,7 +32411,7 @@
         <v>36</v>
       </c>
       <c r="L86" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B86&amp;"'"&amp;","&amp;"'"&amp;C86&amp;"'"&amp;","&amp;VLOOKUP(D86,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E86&amp;","&amp;F86&amp;","&amp;G86&amp;","&amp;H86&amp;","&amp;VLOOKUP(I86,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B86&amp;"'"&amp;","&amp;"'"&amp;C86&amp;"'"&amp;","&amp;VLOOKUP(D86,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E86&amp;","&amp;F86&amp;","&amp;G86&amp;","&amp;H86&amp;","&amp;VLOOKUP(I86,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster081','パワーボルダー',31,144,16,18,0.25,5);</v>
       </c>
     </row>
@@ -32414,7 +32444,7 @@
         <v>36</v>
       </c>
       <c r="L87" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B87&amp;"'"&amp;","&amp;"'"&amp;C87&amp;"'"&amp;","&amp;VLOOKUP(D87,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E87&amp;","&amp;F87&amp;","&amp;G87&amp;","&amp;H87&amp;","&amp;VLOOKUP(I87,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B87&amp;"'"&amp;","&amp;"'"&amp;C87&amp;"'"&amp;","&amp;VLOOKUP(D87,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E87&amp;","&amp;F87&amp;","&amp;G87&amp;","&amp;H87&amp;","&amp;VLOOKUP(I87,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster082','デスボルダー',31,172,20,23,0.25,5);</v>
       </c>
     </row>
@@ -32444,7 +32474,7 @@
         <v>151</v>
       </c>
       <c r="L88" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B88&amp;"'"&amp;","&amp;"'"&amp;C88&amp;"'"&amp;","&amp;VLOOKUP(D88,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E88&amp;","&amp;F88&amp;","&amp;G88&amp;","&amp;H88&amp;","&amp;VLOOKUP(I88,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B88&amp;"'"&amp;","&amp;"'"&amp;C88&amp;"'"&amp;","&amp;VLOOKUP(D88,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E88&amp;","&amp;F88&amp;","&amp;G88&amp;","&amp;H88&amp;","&amp;VLOOKUP(I88,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster083','パンプキンボム',32,130,17,12,0.18,3);</v>
       </c>
     </row>
@@ -32474,7 +32504,7 @@
         <v>151</v>
       </c>
       <c r="L89" s="5" t="str">
-        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B89&amp;"'"&amp;","&amp;"'"&amp;C89&amp;"'"&amp;","&amp;VLOOKUP(D89,コード!$C$48:$I$115,3,FALSE)&amp;","&amp;E89&amp;","&amp;F89&amp;","&amp;G89&amp;","&amp;H89&amp;","&amp;VLOOKUP(I89,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
+        <f>"INSERT INTO m_monster VALUES ("&amp;"'"&amp;B89&amp;"'"&amp;","&amp;"'"&amp;C89&amp;"'"&amp;","&amp;VLOOKUP(D89,コード!$C$48:$I$116,3,FALSE)&amp;","&amp;E89&amp;","&amp;F89&amp;","&amp;G89&amp;","&amp;H89&amp;","&amp;VLOOKUP(I89,コード!$C$5:$I$11,3,FALSE)&amp;");"</f>
         <v>INSERT INTO m_monster VALUES ('monster084','グレネードボム',32,160,24,15,0.2,3);</v>
       </c>
     </row>
@@ -32564,22 +32594,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EB7090A-0065-41E7-85DA-75EEB9504A67}">
   <dimension ref="C3:Q81"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="2" width="7.5" style="5" customWidth="1"/>
-    <col min="3" max="3" width="13.75" style="5" customWidth="1"/>
+    <col min="3" max="3" width="13.69921875" style="5" customWidth="1"/>
     <col min="4" max="4" width="20" style="5" customWidth="1"/>
-    <col min="5" max="5" width="30.625" style="5" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="13.375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="30.59765625" style="5" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="13.3984375" style="5" customWidth="1"/>
     <col min="7" max="7" width="11" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.25" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.75" style="5" customWidth="1"/>
-    <col min="10" max="12" width="9.875" style="18" customWidth="1"/>
-    <col min="13" max="13" width="9.25" style="18" customWidth="1"/>
-    <col min="14" max="14" width="12.625" style="18" customWidth="1"/>
-    <col min="15" max="15" width="27.125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="15.19921875" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.69921875" style="5" customWidth="1"/>
+    <col min="10" max="12" width="9.8984375" style="18" customWidth="1"/>
+    <col min="13" max="13" width="9.19921875" style="18" customWidth="1"/>
+    <col min="14" max="14" width="12.59765625" style="18" customWidth="1"/>
+    <col min="15" max="15" width="27.09765625" style="5" customWidth="1"/>
     <col min="16" max="16" width="7.5" style="5" customWidth="1"/>
-    <col min="17" max="17" width="15.125" style="5" customWidth="1"/>
+    <col min="17" max="17" width="15.09765625" style="5" customWidth="1"/>
     <col min="18" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
@@ -34243,7 +34273,7 @@
         <v>INSERT INTO m_skill VALUES ('skill037','グラビジャ',4,0,0,1,75,50,0.0,1,1200,'現HPの７５％ダメージ');</v>
       </c>
     </row>
-    <row r="41" spans="3:17" ht="40.5">
+    <row r="41" spans="3:17" ht="37.799999999999997">
       <c r="C41" s="47" t="s">
         <v>1048</v>
       </c>
@@ -35995,22 +36025,22 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E63A27D9-C8B6-491D-9205-8D7433312F14}">
   <dimension ref="A4:U522"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="12.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.69921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.8984375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.59765625" style="1" customWidth="1"/>
     <col min="5" max="6" width="9" style="1"/>
-    <col min="7" max="7" width="12.75" style="3" customWidth="1"/>
-    <col min="8" max="8" width="5.375" style="4" customWidth="1"/>
-    <col min="9" max="9" width="14.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.69921875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="5.3984375" style="4" customWidth="1"/>
+    <col min="9" max="9" width="14.09765625" style="1" customWidth="1"/>
     <col min="10" max="11" width="9" style="1"/>
-    <col min="12" max="12" width="17.75" style="1" customWidth="1"/>
+    <col min="12" max="12" width="17.69921875" style="1" customWidth="1"/>
     <col min="13" max="13" width="9" style="1"/>
-    <col min="14" max="14" width="5.25" style="1" customWidth="1"/>
+    <col min="14" max="14" width="5.19921875" style="1" customWidth="1"/>
     <col min="15" max="20" width="9" style="1"/>
-    <col min="21" max="21" width="8.875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="8.8984375" style="1" customWidth="1"/>
     <col min="22" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -52603,7 +52633,7 @@
         <v>INSERT INTO m_monster_skills VALUES ('myskill0505','monster084','skill051',FALSE);</v>
       </c>
     </row>
-    <row r="510" spans="1:21" ht="18.75">
+    <row r="510" spans="1:21" ht="18">
       <c r="A510"/>
       <c r="B510"/>
       <c r="C510"/>
@@ -52626,7 +52656,7 @@
       <c r="T510"/>
       <c r="U510"/>
     </row>
-    <row r="511" spans="1:21" ht="18.75">
+    <row r="511" spans="1:21" ht="18">
       <c r="A511"/>
       <c r="B511"/>
       <c r="C511"/>
@@ -52649,7 +52679,7 @@
       <c r="T511"/>
       <c r="U511"/>
     </row>
-    <row r="512" spans="1:21" ht="18.75">
+    <row r="512" spans="1:21" ht="18">
       <c r="A512"/>
       <c r="B512"/>
       <c r="C512"/>
@@ -52672,7 +52702,7 @@
       <c r="T512"/>
       <c r="U512"/>
     </row>
-    <row r="513" spans="1:21" ht="18.75">
+    <row r="513" spans="1:21" ht="18">
       <c r="A513"/>
       <c r="B513"/>
       <c r="C513"/>
@@ -52695,7 +52725,7 @@
       <c r="T513"/>
       <c r="U513"/>
     </row>
-    <row r="514" spans="1:21" ht="18.75">
+    <row r="514" spans="1:21" ht="18">
       <c r="A514"/>
       <c r="B514"/>
       <c r="C514"/>
@@ -52718,7 +52748,7 @@
       <c r="T514"/>
       <c r="U514"/>
     </row>
-    <row r="515" spans="1:21" ht="18.75">
+    <row r="515" spans="1:21" ht="18">
       <c r="A515"/>
       <c r="B515"/>
       <c r="C515"/>
@@ -52741,7 +52771,7 @@
       <c r="T515"/>
       <c r="U515"/>
     </row>
-    <row r="516" spans="1:21" ht="18.75">
+    <row r="516" spans="1:21" ht="18">
       <c r="A516"/>
       <c r="B516"/>
       <c r="C516"/>
@@ -52764,7 +52794,7 @@
       <c r="T516"/>
       <c r="U516"/>
     </row>
-    <row r="517" spans="1:21" ht="18.75">
+    <row r="517" spans="1:21" ht="18">
       <c r="A517"/>
       <c r="B517"/>
       <c r="C517"/>
@@ -52787,7 +52817,7 @@
       <c r="T517"/>
       <c r="U517"/>
     </row>
-    <row r="518" spans="1:21" ht="18.75">
+    <row r="518" spans="1:21" ht="18">
       <c r="A518"/>
       <c r="B518"/>
       <c r="C518"/>
@@ -52810,7 +52840,7 @@
       <c r="T518"/>
       <c r="U518"/>
     </row>
-    <row r="519" spans="1:21" ht="18.75">
+    <row r="519" spans="1:21" ht="18">
       <c r="A519"/>
       <c r="B519"/>
       <c r="C519"/>
@@ -52833,7 +52863,7 @@
       <c r="T519"/>
       <c r="U519"/>
     </row>
-    <row r="520" spans="1:21" ht="18.75">
+    <row r="520" spans="1:21" ht="18">
       <c r="A520"/>
       <c r="B520"/>
       <c r="C520"/>
@@ -52856,7 +52886,7 @@
       <c r="T520"/>
       <c r="U520"/>
     </row>
-    <row r="521" spans="1:21" ht="18.75">
+    <row r="521" spans="1:21" ht="18">
       <c r="A521"/>
       <c r="B521"/>
       <c r="C521"/>
@@ -52879,7 +52909,7 @@
       <c r="T521"/>
       <c r="U521"/>
     </row>
-    <row r="522" spans="1:21" ht="18.75">
+    <row r="522" spans="1:21" ht="18">
       <c r="A522"/>
       <c r="B522"/>
       <c r="C522"/>
@@ -52911,15 +52941,15 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A843E7EA-D614-495E-86B7-D31F628C6221}">
   <dimension ref="A1:I30"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="1" width="9" style="5"/>
-    <col min="2" max="3" width="17.25" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="17.19921875" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.625" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.75" style="5" customWidth="1"/>
+    <col min="5" max="5" width="11.59765625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.69921875" style="5" customWidth="1"/>
     <col min="7" max="7" width="13.5" style="5" customWidth="1"/>
-    <col min="8" max="8" width="11.875" style="5" customWidth="1"/>
+    <col min="8" max="8" width="11.8984375" style="5" customWidth="1"/>
     <col min="9" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
@@ -53280,13 +53310,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FE71EC6-0DD3-461C-A8FC-74E22154B7A5}">
   <dimension ref="A4:H13"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.6"/>
   <cols>
-    <col min="1" max="1" width="3.875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.8984375" style="1" customWidth="1"/>
     <col min="2" max="6" width="9" style="1"/>
-    <col min="7" max="7" width="4.25" style="1" customWidth="1"/>
-    <col min="8" max="8" width="95.25" style="1" customWidth="1"/>
-    <col min="9" max="9" width="11.875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="4.19921875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="95.19921875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="11.8984375" style="1" customWidth="1"/>
     <col min="10" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>

</xml_diff>